<commit_message>
Temporalidad, arreglo de kpi 09 e implementación kpi 01
</commit_message>
<xml_diff>
--- a/2026/kpis_diarios.xlsx
+++ b/2026/kpis_diarios.xlsx
@@ -506,7 +506,7 @@
         <v>0.6161938064680055</v>
       </c>
       <c r="G2" t="n">
-        <v>20.84603843103255</v>
+        <v>15.90800111938989</v>
       </c>
       <c r="H2" t="n">
         <v>0.5900179384633555</v>
@@ -540,7 +540,7 @@
         <v>0.4962205402149751</v>
       </c>
       <c r="G3" t="n">
-        <v>20.22036671135641</v>
+        <v>13.59540608987651</v>
       </c>
       <c r="H3" t="n">
         <v>0.6733162906341628</v>
@@ -574,7 +574,7 @@
         <v>0.658579893388008</v>
       </c>
       <c r="G4" t="n">
-        <v>39.40461165648725</v>
+        <v>33.28436598191306</v>
       </c>
       <c r="H4" t="n">
         <v>0.5891770578240783</v>
@@ -608,7 +608,7 @@
         <v>0.3752079583333437</v>
       </c>
       <c r="G5" t="n">
-        <v>20.42629762053369</v>
+        <v>16.15640385847833</v>
       </c>
       <c r="H5" t="n">
         <v>0.5042261904241331</v>
@@ -642,7 +642,7 @@
         <v>0.6271687033867497</v>
       </c>
       <c r="G6" t="n">
-        <v>31.15546941153515</v>
+        <v>24.67458872735531</v>
       </c>
       <c r="H6" t="n">
         <v>0.3951512670149406</v>
@@ -676,7 +676,7 @@
         <v>0.8186406817820124</v>
       </c>
       <c r="G7" t="n">
-        <v>41.30553296523806</v>
+        <v>33.76170455703105</v>
       </c>
       <c r="H7" t="n">
         <v>0.3462780709597542</v>
@@ -710,7 +710,7 @@
         <v>0.5974050311232658</v>
       </c>
       <c r="G8" t="n">
-        <v>17.08789110187781</v>
+        <v>12.7397695414339</v>
       </c>
       <c r="H8" t="n">
         <v>0.5381577505889946</v>
@@ -744,7 +744,7 @@
         <v>0.6362348662135183</v>
       </c>
       <c r="G9" t="n">
-        <v>20.74943036786532</v>
+        <v>15.67154484079036</v>
       </c>
       <c r="H9" t="n">
         <v>0.55987263106872</v>
@@ -778,7 +778,7 @@
         <v>0.6002278572538201</v>
       </c>
       <c r="G10" t="n">
-        <v>20.80880930529371</v>
+        <v>15.89034834062051</v>
       </c>
       <c r="H10" t="n">
         <v>0.599789437992314</v>
@@ -812,7 +812,7 @@
         <v>0.4155692666934947</v>
       </c>
       <c r="G11" t="n">
-        <v>15.61604902325549</v>
+        <v>11.96446304564717</v>
       </c>
       <c r="H11" t="n">
         <v>0.5630308143636719</v>
@@ -846,7 +846,7 @@
         <v>0.4020555698497478</v>
       </c>
       <c r="G12" t="n">
-        <v>17.64664808049943</v>
+        <v>13.0739987206134</v>
       </c>
       <c r="H12" t="n">
         <v>0.6583412912504013</v>
@@ -880,7 +880,7 @@
         <v>0.5068540000597004</v>
       </c>
       <c r="G13" t="n">
-        <v>14.57210134628429</v>
+        <v>11.3034584112835</v>
       </c>
       <c r="H13" t="n">
         <v>0.8658564767848408</v>
@@ -914,7 +914,7 @@
         <v>0.5109629623039138</v>
       </c>
       <c r="G14" t="n">
-        <v>16.10705396651488</v>
+        <v>12.56355259780136</v>
       </c>
       <c r="H14" t="n">
         <v>0.6590876162317846</v>
@@ -948,7 +948,7 @@
         <v>0.4217776206346099</v>
       </c>
       <c r="G15" t="n">
-        <v>19.16787977372022</v>
+        <v>14.43656395626747</v>
       </c>
       <c r="H15" t="n">
         <v>0.6749016214307737</v>
@@ -982,7 +982,7 @@
         <v>0.6315798369175979</v>
       </c>
       <c r="G16" t="n">
-        <v>21.59639358293746</v>
+        <v>15.99063852011243</v>
       </c>
       <c r="H16" t="n">
         <v>0.6361433438102551</v>
@@ -1016,7 +1016,7 @@
         <v>0.5409373547143517</v>
       </c>
       <c r="G17" t="n">
-        <v>17.89473854074735</v>
+        <v>13.3787095358836</v>
       </c>
       <c r="H17" t="n">
         <v>0.8272077729846495</v>
@@ -1050,7 +1050,7 @@
         <v>0.5877218059729266</v>
       </c>
       <c r="G18" t="n">
-        <v>18.48034880781057</v>
+        <v>14.13214559966201</v>
       </c>
       <c r="H18" t="n">
         <v>0.6016351404139554</v>
@@ -1084,7 +1084,7 @@
         <v>0.403060064127064</v>
       </c>
       <c r="G19" t="n">
-        <v>18.11888331129509</v>
+        <v>13.71761854569402</v>
       </c>
       <c r="H19" t="n">
         <v>0.6774980676619847</v>
@@ -1118,7 +1118,7 @@
         <v>0.5400947879669654</v>
       </c>
       <c r="G20" t="n">
-        <v>13.93449388202233</v>
+        <v>10.71626828804316</v>
       </c>
       <c r="H20" t="n">
         <v>0.8356605808949387</v>
@@ -1152,7 +1152,7 @@
         <v>0.5587092297069479</v>
       </c>
       <c r="G21" t="n">
-        <v>14.32181108810068</v>
+        <v>10.62214875247648</v>
       </c>
       <c r="H21" t="n">
         <v>0.8941024889114946</v>
@@ -1186,7 +1186,7 @@
         <v>0.4138807863701217</v>
       </c>
       <c r="G22" t="n">
-        <v>17.48646234143725</v>
+        <v>12.96722294740385</v>
       </c>
       <c r="H22" t="n">
         <v>0.7302305504460215</v>
@@ -1220,7 +1220,7 @@
         <v>0.657270307616223</v>
       </c>
       <c r="G23" t="n">
-        <v>22.21869630895036</v>
+        <v>17.09011010079759</v>
       </c>
       <c r="H23" t="n">
         <v>0.5998344670607249</v>
@@ -1254,7 +1254,7 @@
         <v>0.4562410137242582</v>
       </c>
       <c r="G24" t="n">
-        <v>18.45058585698759</v>
+        <v>13.7208412625056</v>
       </c>
       <c r="H24" t="n">
         <v>0.773379355438863</v>
@@ -1288,7 +1288,7 @@
         <v>0.6100759895075983</v>
       </c>
       <c r="G25" t="n">
-        <v>17.9278242528486</v>
+        <v>13.36336848200629</v>
       </c>
       <c r="H25" t="n">
         <v>0.6472136221539632</v>
@@ -1322,7 +1322,7 @@
         <v>0.3963436686992338</v>
       </c>
       <c r="G26" t="n">
-        <v>19.35084194591357</v>
+        <v>14.6717377941612</v>
       </c>
       <c r="H26" t="n">
         <v>0.6764378442343523</v>
@@ -1356,7 +1356,7 @@
         <v>0.3526500511327659</v>
       </c>
       <c r="G27" t="n">
-        <v>21.07392255113966</v>
+        <v>16.35774610467822</v>
       </c>
       <c r="H27" t="n">
         <v>0.860314352164035</v>
@@ -1390,7 +1390,7 @@
         <v>0.8444865234273459</v>
       </c>
       <c r="G28" t="n">
-        <v>41.15885670990488</v>
+        <v>33.03727637489281</v>
       </c>
       <c r="H28" t="n">
         <v>0.8278785846958959</v>
@@ -1424,7 +1424,7 @@
         <v>0.6154103105371432</v>
       </c>
       <c r="G29" t="n">
-        <v>19.6464819754076</v>
+        <v>14.76916173869327</v>
       </c>
       <c r="H29" t="n">
         <v>0.6526517774857234</v>
@@ -1458,7 +1458,7 @@
         <v>0.6568903723501734</v>
       </c>
       <c r="G30" t="n">
-        <v>21.9228102150497</v>
+        <v>16.37742445213249</v>
       </c>
       <c r="H30" t="n">
         <v>0.6904366976631247</v>
@@ -1492,7 +1492,7 @@
         <v>0.4142920473148049</v>
       </c>
       <c r="G31" t="n">
-        <v>17.61508955323155</v>
+        <v>13.3468652606661</v>
       </c>
       <c r="H31" t="n">
         <v>0.7120181727164043</v>
@@ -1526,7 +1526,7 @@
         <v>0.7067345326178629</v>
       </c>
       <c r="G32" t="n">
-        <v>22.28383643698744</v>
+        <v>19.86080041125803</v>
       </c>
       <c r="H32" t="n">
         <v>0.681031476124214</v>
@@ -1560,7 +1560,7 @@
         <v>0.5494150220938279</v>
       </c>
       <c r="G33" t="n">
-        <v>17.26313296054669</v>
+        <v>12.857287798418</v>
       </c>
       <c r="H33" t="n">
         <v>0.3070194917621241</v>
@@ -1594,7 +1594,7 @@
         <v>0.5087939187866138</v>
       </c>
       <c r="G34" t="n">
-        <v>13.97233536933921</v>
+        <v>10.06752712024881</v>
       </c>
       <c r="H34" t="n">
         <v>0.3352629193464599</v>
@@ -1628,7 +1628,7 @@
         <v>0.5145582841002388</v>
       </c>
       <c r="G35" t="n">
-        <v>14.21395638854427</v>
+        <v>9.659820325829726</v>
       </c>
       <c r="H35" t="n">
         <v>0.3100655725316754</v>
@@ -1662,7 +1662,7 @@
         <v>0.5178748498154537</v>
       </c>
       <c r="G36" t="n">
-        <v>15.26054368747207</v>
+        <v>11.22517412929457</v>
       </c>
       <c r="H36" t="n">
         <v>0.3255181430739436</v>
@@ -1696,7 +1696,7 @@
         <v>0.5040184048756827</v>
       </c>
       <c r="G37" t="n">
-        <v>20.57079665562074</v>
+        <v>15.31777084331644</v>
       </c>
       <c r="H37" t="n">
         <v>0.3283830356542376</v>
@@ -1730,7 +1730,7 @@
         <v>0.6439485639513477</v>
       </c>
       <c r="G38" t="n">
-        <v>33.94888881724976</v>
+        <v>27.06773866563281</v>
       </c>
       <c r="H38" t="n">
         <v>0.3162625097467864</v>
@@ -1764,7 +1764,7 @@
         <v>0.5561092380315821</v>
       </c>
       <c r="G39" t="n">
-        <v>18.62526486209337</v>
+        <v>13.48928241716261</v>
       </c>
       <c r="H39" t="n">
         <v>0.3155352305046044</v>
@@ -1798,7 +1798,7 @@
         <v>0.547991086660173</v>
       </c>
       <c r="G40" t="n">
-        <v>16.44135730872285</v>
+        <v>11.74684649131636</v>
       </c>
       <c r="H40" t="n">
         <v>0.2879482448143477</v>
@@ -1832,7 +1832,7 @@
         <v>0.5232281363995368</v>
       </c>
       <c r="G41" t="n">
-        <v>16.28503627281709</v>
+        <v>11.94225117562778</v>
       </c>
       <c r="H41" t="n">
         <v>0.2863628080971266</v>
@@ -1866,7 +1866,7 @@
         <v>0.6080846067733948</v>
       </c>
       <c r="G42" t="n">
-        <v>18.51338700297904</v>
+        <v>13.1521900339564</v>
       </c>
       <c r="H42" t="n">
         <v>0.3176562917936633</v>
@@ -1900,7 +1900,7 @@
         <v>0.5083177194653514</v>
       </c>
       <c r="G43" t="n">
-        <v>15.66569087849687</v>
+        <v>11.32409372952436</v>
       </c>
       <c r="H43" t="n">
         <v>0.2984232125206857</v>
@@ -1934,7 +1934,7 @@
         <v>0.4613653039490254</v>
       </c>
       <c r="G44" t="n">
-        <v>22.45484518394695</v>
+        <v>17.4481253433728</v>
       </c>
       <c r="H44" t="n">
         <v>0.3505202895569106</v>
@@ -1968,7 +1968,7 @@
         <v>0.475261624574809</v>
       </c>
       <c r="G45" t="n">
-        <v>31.76830840316199</v>
+        <v>25.5535219304126</v>
       </c>
       <c r="H45" t="n">
         <v>0.1458011068256753</v>
@@ -2002,7 +2002,7 @@
         <v>0.5005091573843278</v>
       </c>
       <c r="G46" t="n">
-        <v>16.00143228419213</v>
+        <v>11.65631184039025</v>
       </c>
       <c r="H46" t="n">
         <v>0.3406828815997597</v>
@@ -2036,7 +2036,7 @@
         <v>0.5609146915711951</v>
       </c>
       <c r="G47" t="n">
-        <v>17.92288304446027</v>
+        <v>13.12313968961564</v>
       </c>
       <c r="H47" t="n">
         <v>0.2875647679242391</v>
@@ -2070,7 +2070,7 @@
         <v>0.5676093111311565</v>
       </c>
       <c r="G48" t="n">
-        <v>17.09304028647021</v>
+        <v>12.88143940708193</v>
       </c>
       <c r="H48" t="n">
         <v>0.3156801644945513</v>
@@ -2104,7 +2104,7 @@
         <v>0.5527255843065874</v>
       </c>
       <c r="G49" t="n">
-        <v>16.87536045051807</v>
+        <v>12.33516856552613</v>
       </c>
       <c r="H49" t="n">
         <v>0.3168487972811664</v>
@@ -2138,7 +2138,7 @@
         <v>0.5974504653290019</v>
       </c>
       <c r="G50" t="n">
-        <v>17.78765406659607</v>
+        <v>13.23988302824455</v>
       </c>
       <c r="H50" t="n">
         <v>0.3270922924681754</v>
@@ -2172,7 +2172,7 @@
         <v>0.4843754492768066</v>
       </c>
       <c r="G51" t="n">
-        <v>19.47701031070291</v>
+        <v>14.68065767736155</v>
       </c>
       <c r="H51" t="n">
         <v>0.3118033544542869</v>
@@ -2206,7 +2206,7 @@
         <v>0.6245303272382846</v>
       </c>
       <c r="G52" t="n">
-        <v>33.70912175646203</v>
+        <v>27.05611663225597</v>
       </c>
       <c r="H52" t="n">
         <v>0.3167185257533623</v>
@@ -2240,7 +2240,7 @@
         <v>0.5502713268171853</v>
       </c>
       <c r="G53" t="n">
-        <v>16.65127627915144</v>
+        <v>12.02366944851133</v>
       </c>
       <c r="H53" t="n">
         <v>0.3145242223788963</v>
@@ -2274,7 +2274,7 @@
         <v>0.5493460081569158</v>
       </c>
       <c r="G54" t="n">
-        <v>16.30711161341631</v>
+        <v>11.59278208836471</v>
       </c>
       <c r="H54" t="n">
         <v>0.3082713472314411</v>
@@ -2308,7 +2308,7 @@
         <v>0.5714506114256933</v>
       </c>
       <c r="G55" t="n">
-        <v>16.00018902571915</v>
+        <v>11.72408791706035</v>
       </c>
       <c r="H55" t="n">
         <v>0.3003961487425322</v>
@@ -2342,7 +2342,7 @@
         <v>0.5856974999377869</v>
       </c>
       <c r="G56" t="n">
-        <v>17.87801815890438</v>
+        <v>13.05339459369789</v>
       </c>
       <c r="H56" t="n">
         <v>0.3035019710367688</v>
@@ -2376,7 +2376,7 @@
         <v>0.6029364342821907</v>
       </c>
       <c r="G57" t="n">
-        <v>16.80574132436693</v>
+        <v>12.26213827091041</v>
       </c>
       <c r="H57" t="n">
         <v>0.3221987740304654</v>
@@ -2410,7 +2410,7 @@
         <v>0.4737528142595747</v>
       </c>
       <c r="G58" t="n">
-        <v>20.26080620733605</v>
+        <v>15.48696833111345</v>
       </c>
       <c r="H58" t="n">
         <v>0.3024483218963998</v>
@@ -2444,7 +2444,7 @@
         <v>0.5399782221275068</v>
       </c>
       <c r="G59" t="n">
-        <v>32.69117545702223</v>
+        <v>25.77696361299702</v>
       </c>
       <c r="H59" t="n">
         <v>0.3267088890415784</v>
@@ -2478,7 +2478,7 @@
         <v>0.5629584253230356</v>
       </c>
       <c r="G60" t="n">
-        <v>16.14977829351245</v>
+        <v>11.95561241172095</v>
       </c>
       <c r="H60" t="n">
         <v>0.3190014644560187</v>
@@ -2512,7 +2512,7 @@
         <v>0.6144440557512296</v>
       </c>
       <c r="G61" t="n">
-        <v>16.67613849041776</v>
+        <v>12.11987710703879</v>
       </c>
       <c r="H61" t="n">
         <v>0.3036518516741798</v>
@@ -2546,7 +2546,7 @@
         <v>0.5560522785285866</v>
       </c>
       <c r="G62" t="n">
-        <v>17.13394528042179</v>
+        <v>12.9158146027168</v>
       </c>
       <c r="H62" t="n">
         <v>0.307889380127285</v>
@@ -2580,7 +2580,7 @@
         <v>0.6094522485474075</v>
       </c>
       <c r="G63" t="n">
-        <v>17.78028252428921</v>
+        <v>14.56251993026877</v>
       </c>
       <c r="H63" t="n">
         <v>0.3059610621088545</v>
@@ -2974,7 +2974,7 @@
         <v>0.5382770994741621</v>
       </c>
       <c r="G84" t="n">
-        <v>6.227928988394337</v>
+        <v>3.714717982524127</v>
       </c>
       <c r="H84" t="n">
         <v>0.325042602187893</v>
@@ -3008,7 +3008,7 @@
         <v>0.5684309510642604</v>
       </c>
       <c r="G85" t="n">
-        <v>14.33704210097863</v>
+        <v>10.339583597473</v>
       </c>
       <c r="H85" t="n">
         <v>0.3495482102275561</v>
@@ -3042,7 +3042,7 @@
         <v>0.5800679937333191</v>
       </c>
       <c r="G86" t="n">
-        <v>14.75384271112838</v>
+        <v>10.85250054467341</v>
       </c>
       <c r="H86" t="n">
         <v>0.3407167022864599</v>
@@ -3076,7 +3076,7 @@
         <v>0.5801216015677448</v>
       </c>
       <c r="G87" t="n">
-        <v>14.78377997455162</v>
+        <v>11.23139114482381</v>
       </c>
       <c r="H87" t="n">
         <v>0.3282729447666313</v>
@@ -3110,7 +3110,7 @@
         <v>0.6064997879965585</v>
       </c>
       <c r="G88" t="n">
-        <v>16.03442383306447</v>
+        <v>11.51736117555344</v>
       </c>
       <c r="H88" t="n">
         <v>0.3331267788208969</v>
@@ -3144,7 +3144,7 @@
         <v>0.4303142567135341</v>
       </c>
       <c r="G89" t="n">
-        <v>22.66709900457411</v>
+        <v>17.97116489982409</v>
       </c>
       <c r="H89" t="n">
         <v>0.3551678725961598</v>
@@ -3178,7 +3178,7 @@
         <v>0.666393410025643</v>
       </c>
       <c r="G90" t="n">
-        <v>40.53843951129422</v>
+        <v>33.47544279442169</v>
       </c>
       <c r="H90" t="n">
         <v>0.4060548097686967</v>
@@ -3212,7 +3212,7 @@
         <v>0.5859569333302459</v>
       </c>
       <c r="G91" t="n">
-        <v>15.78863058166576</v>
+        <v>11.74543975189895</v>
       </c>
       <c r="H91" t="n">
         <v>0.3116391034742668</v>
@@ -3246,7 +3246,7 @@
         <v>0.5702246466770401</v>
       </c>
       <c r="G92" t="n">
-        <v>14.52447406051968</v>
+        <v>10.73112374449039</v>
       </c>
       <c r="H92" t="n">
         <v>0.3182447273147485</v>
@@ -3280,7 +3280,7 @@
         <v>0.5894561332488307</v>
       </c>
       <c r="G93" t="n">
-        <v>14.88300289526948</v>
+        <v>11.05177654726302</v>
       </c>
       <c r="H93" t="n">
         <v>0.326601560878495</v>
@@ -3314,7 +3314,7 @@
         <v>0.6560936285863271</v>
       </c>
       <c r="G94" t="n">
-        <v>15.00938083220894</v>
+        <v>12.34256507372057</v>
       </c>
       <c r="H94" t="n">
         <v>0.2898436177501996</v>
@@ -3348,7 +3348,7 @@
         <v>0.4661064728370691</v>
       </c>
       <c r="G95" t="n">
-        <v>25.63788778551184</v>
+        <v>18.35116361960831</v>
       </c>
       <c r="H95" t="n">
         <v>0.4689050061774496</v>
@@ -3382,7 +3382,7 @@
         <v>0.509097848776623</v>
       </c>
       <c r="G96" t="n">
-        <v>23.16146356859822</v>
+        <v>16.66473294705898</v>
       </c>
       <c r="H96" t="n">
         <v>0.5001341058694054</v>
@@ -3416,7 +3416,7 @@
         <v>0.47625389129275</v>
       </c>
       <c r="G97" t="n">
-        <v>23.03450631852137</v>
+        <v>16.30248309240607</v>
       </c>
       <c r="H97" t="n">
         <v>0.4680956584811089</v>
@@ -3450,7 +3450,7 @@
         <v>0.6397998292629419</v>
       </c>
       <c r="G98" t="n">
-        <v>20.56301078824371</v>
+        <v>14.63715044740583</v>
       </c>
       <c r="H98" t="n">
         <v>0.5018423552388409</v>
@@ -3484,7 +3484,7 @@
         <v>0.6034673943207256</v>
       </c>
       <c r="G99" t="n">
-        <v>23.45726213778209</v>
+        <v>16.73121081400487</v>
       </c>
       <c r="H99" t="n">
         <v>0.4688014901441235</v>
@@ -3518,7 +3518,7 @@
         <v>0.9371530601218309</v>
       </c>
       <c r="G100" t="n">
-        <v>37.83167752721206</v>
+        <v>30.7580143488751</v>
       </c>
       <c r="H100" t="n">
         <v>0.4233972762038309</v>
@@ -3552,7 +3552,7 @@
         <v>0.5316154255684278</v>
       </c>
       <c r="G101" t="n">
-        <v>34.15666456085506</v>
+        <v>27.46556340085986</v>
       </c>
       <c r="H101" t="n">
         <v>0.4666267251275778</v>
@@ -3586,7 +3586,7 @@
         <v>0.5627701876669082</v>
       </c>
       <c r="G102" t="n">
-        <v>21.78207311293708</v>
+        <v>14.3275787355833</v>
       </c>
       <c r="H102" t="n">
         <v>0.4586857693859554</v>
@@ -3620,7 +3620,7 @@
         <v>0.5653189199803762</v>
       </c>
       <c r="G103" t="n">
-        <v>19.87316298206582</v>
+        <v>13.11409759986261</v>
       </c>
       <c r="H103" t="n">
         <v>0.4521450977332102</v>
@@ -3654,7 +3654,7 @@
         <v>0.4874200002046397</v>
       </c>
       <c r="G104" t="n">
-        <v>22.94050351991925</v>
+        <v>16.43726673288388</v>
       </c>
       <c r="H104" t="n">
         <v>0.4853416514342039</v>
@@ -3688,7 +3688,7 @@
         <v>0.4846875621168092</v>
       </c>
       <c r="G105" t="n">
-        <v>23.02728599791975</v>
+        <v>15.75500556892712</v>
       </c>
       <c r="H105" t="n">
         <v>0.4593679008060755</v>
@@ -3722,7 +3722,7 @@
         <v>0.7295172305148961</v>
       </c>
       <c r="G106" t="n">
-        <v>31.11977262575841</v>
+        <v>25.2641109032744</v>
       </c>
       <c r="H106" t="n">
         <v>0.4147236514388081</v>
@@ -3756,7 +3756,7 @@
         <v>0.8835910227414981</v>
       </c>
       <c r="G107" t="n">
-        <v>36.85000705958244</v>
+        <v>30.19044807220596</v>
       </c>
       <c r="H107" t="n">
         <v>0.1792139947716758</v>
@@ -3790,7 +3790,7 @@
         <v>0.4739223179493989</v>
       </c>
       <c r="G108" t="n">
-        <v>26.81163901904251</v>
+        <v>18.28534667735214</v>
       </c>
       <c r="H108" t="n">
         <v>0.4605918559915958</v>
@@ -3824,7 +3824,7 @@
         <v>0.5979244828507967</v>
       </c>
       <c r="G109" t="n">
-        <v>25.18632556446886</v>
+        <v>17.12891356938725</v>
       </c>
       <c r="H109" t="n">
         <v>0.4508519814092022</v>
@@ -3858,7 +3858,7 @@
         <v>0.5075761131997438</v>
       </c>
       <c r="G110" t="n">
-        <v>22.53867996233758</v>
+        <v>15.91536108945917</v>
       </c>
       <c r="H110" t="n">
         <v>0.4879386819775229</v>
@@ -3892,7 +3892,7 @@
         <v>0.4869873769036537</v>
       </c>
       <c r="G111" t="n">
-        <v>21.51932780690131</v>
+        <v>15.7571078522099</v>
       </c>
       <c r="H111" t="n">
         <v>0.5229979270177876</v>
@@ -3926,7 +3926,7 @@
         <v>0.5486937381128525</v>
       </c>
       <c r="G112" t="n">
-        <v>17.20433902048802</v>
+        <v>12.27657854911584</v>
       </c>
       <c r="H112" t="n">
         <v>0.4766489333717598</v>
@@ -3960,7 +3960,7 @@
         <v>0.6515572685078656</v>
       </c>
       <c r="G113" t="n">
-        <v>26.9761734083805</v>
+        <v>21.59216846320603</v>
       </c>
       <c r="H113" t="n">
         <v>0.4496603659672637</v>
@@ -3994,7 +3994,7 @@
         <v>0.8343838137276556</v>
       </c>
       <c r="G114" t="n">
-        <v>35.57794414040371</v>
+        <v>28.05212453590654</v>
       </c>
       <c r="H114" t="n">
         <v>0.4914874537237948</v>
@@ -4028,7 +4028,7 @@
         <v>0.517278725195747</v>
       </c>
       <c r="G115" t="n">
-        <v>20.33728046471892</v>
+        <v>14.01115503493609</v>
       </c>
       <c r="H115" t="n">
         <v>0.470308727942726</v>
@@ -4062,7 +4062,7 @@
         <v>0.5503909048021252</v>
       </c>
       <c r="G116" t="n">
-        <v>20.82089505174066</v>
+        <v>15.31944833177247</v>
       </c>
       <c r="H116" t="n">
         <v>0.4897927010768036</v>
@@ -4096,7 +4096,7 @@
         <v>0.5680349026033883</v>
       </c>
       <c r="G117" t="n">
-        <v>20.64582222301599</v>
+        <v>14.96290701165526</v>
       </c>
       <c r="H117" t="n">
         <v>0.4716440311374074</v>
@@ -4130,7 +4130,7 @@
         <v>0.5257011473821512</v>
       </c>
       <c r="G118" t="n">
-        <v>22.10537737817858</v>
+        <v>15.86304670130096</v>
       </c>
       <c r="H118" t="n">
         <v>0.4886101886244908</v>
@@ -4164,7 +4164,7 @@
         <v>0.512049930928401</v>
       </c>
       <c r="G119" t="n">
-        <v>23.94359098696643</v>
+        <v>16.69429599392691</v>
       </c>
       <c r="H119" t="n">
         <v>0.5110595964074768</v>
@@ -4198,7 +4198,7 @@
         <v>0.6384032015415748</v>
       </c>
       <c r="G120" t="n">
-        <v>25.39200909654478</v>
+        <v>18.41089539920545</v>
       </c>
       <c r="H120" t="n">
         <v>0.4137058587641798</v>
@@ -4232,7 +4232,7 @@
         <v>0.7652803592965226</v>
       </c>
       <c r="G121" t="n">
-        <v>22.87841898470264</v>
+        <v>17.87078215527818</v>
       </c>
       <c r="H121" t="n">
         <v>0.4382875627380665</v>
@@ -4266,7 +4266,7 @@
         <v>0.4961458495252349</v>
       </c>
       <c r="G122" t="n">
-        <v>24.18344415179835</v>
+        <v>17.14729408569213</v>
       </c>
       <c r="H122" t="n">
         <v>0.483754920945464</v>
@@ -4300,7 +4300,7 @@
         <v>0.7965749270604372</v>
       </c>
       <c r="G123" t="n">
-        <v>32.29558717068018</v>
+        <v>26.14965147051482</v>
       </c>
       <c r="H123" t="n">
         <v>0.4767874193681105</v>
@@ -4334,7 +4334,7 @@
         <v>0.4928639595673332</v>
       </c>
       <c r="G124" t="n">
-        <v>19.88798693719447</v>
+        <v>13.75726491925134</v>
       </c>
       <c r="H124" t="n">
         <v>0.4474173472968471</v>
@@ -4368,7 +4368,7 @@
         <v>0.4106391382340593</v>
       </c>
       <c r="G125" t="n">
-        <v>22.78280315920176</v>
+        <v>20.7414535611856</v>
       </c>
       <c r="H125" t="n">
         <v>0.4919071646044334</v>
@@ -4402,7 +4402,7 @@
         <v>0.5457270037976798</v>
       </c>
       <c r="G126" t="n">
-        <v>22.99718817822434</v>
+        <v>16.97622748836255</v>
       </c>
       <c r="H126" t="n">
         <v>0.318251351449966</v>
@@ -4436,7 +4436,7 @@
         <v>0.594059136932189</v>
       </c>
       <c r="G127" t="n">
-        <v>23.32644222992283</v>
+        <v>16.88297994883917</v>
       </c>
       <c r="H127" t="n">
         <v>0.2566292604104535</v>
@@ -4470,7 +4470,7 @@
         <v>0.5863809531916907</v>
       </c>
       <c r="G128" t="n">
-        <v>23.09952034930784</v>
+        <v>17.62855964569489</v>
       </c>
       <c r="H128" t="n">
         <v>0.2577120181874319</v>
@@ -4504,7 +4504,7 @@
         <v>0.4840405207757912</v>
       </c>
       <c r="G129" t="n">
-        <v>22.42497443796154</v>
+        <v>17.30021452270166</v>
       </c>
       <c r="H129" t="n">
         <v>0.2915250812972112</v>
@@ -4538,7 +4538,7 @@
         <v>0.6631727867957693</v>
       </c>
       <c r="G130" t="n">
-        <v>28.23464471404134</v>
+        <v>22.19626031584914</v>
       </c>
       <c r="H130" t="n">
         <v>0.352269229493912</v>
@@ -4572,7 +4572,7 @@
         <v>0.4870827790477794</v>
       </c>
       <c r="G131" t="n">
-        <v>28.45721366143221</v>
+        <v>22.01706809789879</v>
       </c>
       <c r="H131" t="n">
         <v>0.33913383598665</v>
@@ -4606,7 +4606,7 @@
         <v>0.495956654404817</v>
       </c>
       <c r="G132" t="n">
-        <v>21.79318991591187</v>
+        <v>15.60090537040209</v>
       </c>
       <c r="H132" t="n">
         <v>0.2820419586876066</v>
@@ -4640,7 +4640,7 @@
         <v>0.6108720740748012</v>
       </c>
       <c r="G133" t="n">
-        <v>23.42852909620887</v>
+        <v>17.73665500287675</v>
       </c>
       <c r="H133" t="n">
         <v>0.2310437426794061</v>
@@ -4674,7 +4674,7 @@
         <v>0.5893874469978847</v>
       </c>
       <c r="G134" t="n">
-        <v>21.73033210054437</v>
+        <v>4.164501788964369</v>
       </c>
       <c r="H134" t="n">
         <v>0.2613754196552219</v>
@@ -4708,7 +4708,7 @@
         <v>0.5445182784121085</v>
       </c>
       <c r="G135" t="n">
-        <v>21.6600464677535</v>
+        <v>15.87192754964333</v>
       </c>
       <c r="H135" t="n">
         <v>0.3187019058905466</v>
@@ -4742,7 +4742,7 @@
         <v>0.5553937657060437</v>
       </c>
       <c r="G136" t="n">
-        <v>21.92302164150179</v>
+        <v>15.8471438009335</v>
       </c>
       <c r="H136" t="n">
         <v>0.2620648859913682</v>
@@ -4776,7 +4776,7 @@
         <v>0.6107858804434196</v>
       </c>
       <c r="G137" t="n">
-        <v>27.64894664458593</v>
+        <v>22.12951226919157</v>
       </c>
       <c r="H137" t="n">
         <v>0.3480285762731958</v>
@@ -4810,7 +4810,7 @@
         <v>0.4884690438100637</v>
       </c>
       <c r="G138" t="n">
-        <v>25.9150981470416</v>
+        <v>27.11879270363876</v>
       </c>
       <c r="H138" t="n">
         <v>0.1467516618445535</v>
@@ -4844,7 +4844,7 @@
         <v>0.5848294550411053</v>
       </c>
       <c r="G139" t="n">
-        <v>21.85288410090162</v>
+        <v>16.05010922773915</v>
       </c>
       <c r="H139" t="n">
         <v>0.274719845632944</v>
@@ -4878,7 +4878,7 @@
         <v>0.5760384439671725</v>
       </c>
       <c r="G140" t="n">
-        <v>25.59358289842987</v>
+        <v>18.66404670125102</v>
       </c>
       <c r="H140" t="n">
         <v>0.3130378308015795</v>
@@ -4912,7 +4912,7 @@
         <v>0.6740821368303995</v>
       </c>
       <c r="G141" t="n">
-        <v>24.25844544715972</v>
+        <v>17.93270519374234</v>
       </c>
       <c r="H141" t="n">
         <v>0.3058999559318509</v>
@@ -4946,7 +4946,7 @@
         <v>0.5385893946534006</v>
       </c>
       <c r="G142" t="n">
-        <v>22.91535522177239</v>
+        <v>17.1635506335462</v>
       </c>
       <c r="H142" t="n">
         <v>0.3160602088984504</v>
@@ -4980,7 +4980,7 @@
         <v>0.5323130614859598</v>
       </c>
       <c r="G143" t="n">
-        <v>20.77411859371524</v>
+        <v>15.06023082251203</v>
       </c>
       <c r="H143" t="n">
         <v>0.297446393972264</v>
@@ -5014,7 +5014,7 @@
         <v>0.5918203964237123</v>
       </c>
       <c r="G144" t="n">
-        <v>26.92234619694752</v>
+        <v>20.72798337956763</v>
       </c>
       <c r="H144" t="n">
         <v>0.3299730413430512</v>
@@ -5048,7 +5048,7 @@
         <v>0.6374348370863907</v>
       </c>
       <c r="G145" t="n">
-        <v>24.61863031138821</v>
+        <v>18.34161991966377</v>
       </c>
       <c r="H145" t="n">
         <v>0.367227031623784</v>
@@ -5082,7 +5082,7 @@
         <v>0.5788029370907951</v>
       </c>
       <c r="G146" t="n">
-        <v>24.00399056243931</v>
+        <v>17.04308622328072</v>
       </c>
       <c r="H146" t="n">
         <v>0.3468025540142716</v>
@@ -5116,7 +5116,7 @@
         <v>0.6416792501949651</v>
       </c>
       <c r="G147" t="n">
-        <v>22.75616791377917</v>
+        <v>16.3469513139805</v>
       </c>
       <c r="H147" t="n">
         <v>0.3265585028568002</v>
@@ -5150,7 +5150,7 @@
         <v>0.5509078690507395</v>
       </c>
       <c r="G148" t="n">
-        <v>20.20776362016118</v>
+        <v>15.07243801326847</v>
       </c>
       <c r="H148" t="n">
         <v>0.2788301264738265</v>
@@ -5184,7 +5184,7 @@
         <v>0.6212272912728295</v>
       </c>
       <c r="G149" t="n">
-        <v>22.89444423167729</v>
+        <v>17.03658838201837</v>
       </c>
       <c r="H149" t="n">
         <v>0.3470120653264258</v>
@@ -5218,7 +5218,7 @@
         <v>0.6457469852737538</v>
       </c>
       <c r="G150" t="n">
-        <v>24.97800581935701</v>
+        <v>18.61289023077958</v>
       </c>
       <c r="H150" t="n">
         <v>0.3134419606832198</v>
@@ -5252,7 +5252,7 @@
         <v>0.6760282560074165</v>
       </c>
       <c r="G151" t="n">
-        <v>23.69037392297219</v>
+        <v>18.43141268177828</v>
       </c>
       <c r="H151" t="n">
         <v>0.3035012794944893</v>
@@ -5286,7 +5286,7 @@
         <v>0.671733726709971</v>
       </c>
       <c r="G152" t="n">
-        <v>29.16614648328469</v>
+        <v>23.13383563351555</v>
       </c>
       <c r="H152" t="n">
         <v>0.3512943089191872</v>
@@ -5320,7 +5320,7 @@
         <v>0.5769115791814141</v>
       </c>
       <c r="G153" t="n">
-        <v>22.97198507621286</v>
+        <v>16.1753967417536</v>
       </c>
       <c r="H153" t="n">
         <v>0.3252614320605496</v>
@@ -5354,7 +5354,7 @@
         <v>0.6065168718519321</v>
       </c>
       <c r="G154" t="n">
-        <v>22.84536728750815</v>
+        <v>15.84688490463757</v>
       </c>
       <c r="H154" t="n">
         <v>0.319648528049321</v>
@@ -5388,7 +5388,7 @@
         <v>0.596607810884258</v>
       </c>
       <c r="G155" t="n">
-        <v>21.99652740433805</v>
+        <v>16.34986976928148</v>
       </c>
       <c r="H155" t="n">
         <v>0.3204701227994584</v>
@@ -5422,7 +5422,7 @@
         <v>0.7271999716794374</v>
       </c>
       <c r="G156" t="n">
-        <v>23.40056719528324</v>
+        <v>19.45369483809652</v>
       </c>
       <c r="H156" t="n">
         <v>0.3340956776003985</v>
@@ -5456,7 +5456,7 @@
         <v>0.5693289225041953</v>
       </c>
       <c r="G157" t="n">
-        <v>14.79429088927939</v>
+        <v>11.07521639835844</v>
       </c>
       <c r="H157" t="n">
         <v>0.3764180224449014</v>
@@ -5490,7 +5490,7 @@
         <v>0.5176115731353013</v>
       </c>
       <c r="G158" t="n">
-        <v>14.57395365895813</v>
+        <v>10.78316172778315</v>
       </c>
       <c r="H158" t="n">
         <v>0.3674624061462096</v>
@@ -5524,7 +5524,7 @@
         <v>0.5329956368121436</v>
       </c>
       <c r="G159" t="n">
-        <v>14.03140102132545</v>
+        <v>10.27307072243949</v>
       </c>
       <c r="H159" t="n">
         <v>0.3299858190578098</v>
@@ -5558,7 +5558,7 @@
         <v>0.5099545218940919</v>
       </c>
       <c r="G160" t="n">
-        <v>14.29516454899591</v>
+        <v>10.47637645585858</v>
       </c>
       <c r="H160" t="n">
         <v>0.3591364464649529</v>
@@ -5592,7 +5592,7 @@
         <v>0.5821764879241202</v>
       </c>
       <c r="G161" t="n">
-        <v>29.4630066712648</v>
+        <v>22.99102921969126</v>
       </c>
       <c r="H161" t="n">
         <v>0.3767643207032148</v>
@@ -5626,7 +5626,7 @@
         <v>0.5080849114786729</v>
       </c>
       <c r="G162" t="n">
-        <v>31.76042124258766</v>
+        <v>25.48989872701862</v>
       </c>
       <c r="H162" t="n">
         <v>0.4233517925526672</v>
@@ -5660,7 +5660,7 @@
         <v>0.5178773504129615</v>
       </c>
       <c r="G163" t="n">
-        <v>13.8624551660022</v>
+        <v>10.35146583471869</v>
       </c>
       <c r="H163" t="n">
         <v>0.3689144991971365</v>
@@ -5694,7 +5694,7 @@
         <v>0.488950894296481</v>
       </c>
       <c r="G164" t="n">
-        <v>13.86006529190484</v>
+        <v>10.14152237741039</v>
       </c>
       <c r="H164" t="n">
         <v>0.3484987232672545</v>
@@ -5728,7 +5728,7 @@
         <v>0.4870085700343633</v>
       </c>
       <c r="G165" t="n">
-        <v>13.97120685473949</v>
+        <v>10.32284814057958</v>
       </c>
       <c r="H165" t="n">
         <v>0.3390582346190428</v>
@@ -5762,7 +5762,7 @@
         <v>0.5368415207462458</v>
       </c>
       <c r="G166" t="n">
-        <v>15.00296150887756</v>
+        <v>11.18193349600317</v>
       </c>
       <c r="H166" t="n">
         <v>0.4001059915153229</v>
@@ -5796,7 +5796,7 @@
         <v>0.4997189355747075</v>
       </c>
       <c r="G167" t="n">
-        <v>15.19491015359701</v>
+        <v>11.40347567502216</v>
       </c>
       <c r="H167" t="n">
         <v>0.3327557886298957</v>
@@ -5830,7 +5830,7 @@
         <v>0.4660604098447629</v>
       </c>
       <c r="G168" t="n">
-        <v>25.37087132038504</v>
+        <v>20.01233532208784</v>
       </c>
       <c r="H168" t="n">
         <v>0.3754062537365634</v>
@@ -5864,7 +5864,7 @@
         <v>0.5443179506370245</v>
       </c>
       <c r="G169" t="n">
-        <v>33.26779459826077</v>
+        <v>26.50125880950029</v>
       </c>
       <c r="H169" t="n">
         <v>0.141449985052422</v>
@@ -5898,7 +5898,7 @@
         <v>0.5441647163594464</v>
       </c>
       <c r="G170" t="n">
-        <v>15.05133077287844</v>
+        <v>10.8248790003379</v>
       </c>
       <c r="H170" t="n">
         <v>0.3388629881132731</v>
@@ -5932,7 +5932,7 @@
         <v>0.5420104392196332</v>
       </c>
       <c r="G171" t="n">
-        <v>15.32427272768756</v>
+        <v>11.21627590200817</v>
       </c>
       <c r="H171" t="n">
         <v>0.3819370624383091</v>
@@ -5966,7 +5966,7 @@
         <v>0.5184345936718225</v>
       </c>
       <c r="G172" t="n">
-        <v>15.02163763067953</v>
+        <v>11.03347340829645</v>
       </c>
       <c r="H172" t="n">
         <v>0.3610876975817425</v>
@@ -6000,7 +6000,7 @@
         <v>0.4930040502462394</v>
       </c>
       <c r="G173" t="n">
-        <v>14.80690750731429</v>
+        <v>10.9657280963408</v>
       </c>
       <c r="H173" t="n">
         <v>0.3646310757635193</v>
@@ -6034,7 +6034,7 @@
         <v>0.5248100023571133</v>
       </c>
       <c r="G174" t="n">
-        <v>15.71560481430441</v>
+        <v>11.7107899489524</v>
       </c>
       <c r="H174" t="n">
         <v>0.3459224004655481</v>
@@ -6068,7 +6068,7 @@
         <v>0.4869724579882283</v>
       </c>
       <c r="G175" t="n">
-        <v>25.86575387359807</v>
+        <v>20.07569221172079</v>
       </c>
       <c r="H175" t="n">
         <v>0.3741440704244816</v>
@@ -6102,7 +6102,7 @@
         <v>0.5839839992729386</v>
       </c>
       <c r="G176" t="n">
-        <v>32.71505435408679</v>
+        <v>26.00963554527753</v>
       </c>
       <c r="H176" t="n">
         <v>0.4127623020333381</v>
@@ -6136,7 +6136,7 @@
         <v>0.5149372913123929</v>
       </c>
       <c r="G177" t="n">
-        <v>14.52884385856742</v>
+        <v>10.78466710815911</v>
       </c>
       <c r="H177" t="n">
         <v>0.3974016516263739</v>
@@ -6170,7 +6170,7 @@
         <v>0.4727874996467325</v>
       </c>
       <c r="G178" t="n">
-        <v>13.80999908717407</v>
+        <v>10.39966708267917</v>
       </c>
       <c r="H178" t="n">
         <v>0.4026585050609974</v>
@@ -6204,7 +6204,7 @@
         <v>0.5545763119501259</v>
       </c>
       <c r="G179" t="n">
-        <v>15.23771314998396</v>
+        <v>11.17946170389634</v>
       </c>
       <c r="H179" t="n">
         <v>0.3770954515477949</v>
@@ -6238,7 +6238,7 @@
         <v>0.5314937549656935</v>
       </c>
       <c r="G180" t="n">
-        <v>15.51683316695505</v>
+        <v>11.56957632799917</v>
       </c>
       <c r="H180" t="n">
         <v>0.3958733096761459</v>
@@ -6272,7 +6272,7 @@
         <v>0.4664685837875094</v>
       </c>
       <c r="G181" t="n">
-        <v>15.3172513981406</v>
+        <v>11.48487012837157</v>
       </c>
       <c r="H181" t="n">
         <v>0.4081384154545797</v>
@@ -6306,7 +6306,7 @@
         <v>0.5484516252450201</v>
       </c>
       <c r="G182" t="n">
-        <v>30.34667799900044</v>
+        <v>24.41094441165811</v>
       </c>
       <c r="H182" t="n">
         <v>0.3735120655474011</v>
@@ -6340,7 +6340,7 @@
         <v>0.5648728421473431</v>
       </c>
       <c r="G183" t="n">
-        <v>33.24519540719721</v>
+        <v>26.36972900155338</v>
       </c>
       <c r="H183" t="n">
         <v>0.4185385465060851</v>
@@ -6374,7 +6374,7 @@
         <v>0.5110525599243713</v>
       </c>
       <c r="G184" t="n">
-        <v>14.5534718632863</v>
+        <v>10.71558105452063</v>
       </c>
       <c r="H184" t="n">
         <v>0.3773740935398499</v>
@@ -6408,7 +6408,7 @@
         <v>0.4485470738623258</v>
       </c>
       <c r="G185" t="n">
-        <v>13.78941800527537</v>
+        <v>10.17179371932394</v>
       </c>
       <c r="H185" t="n">
         <v>0.3868851539965473</v>
@@ -6442,7 +6442,7 @@
         <v>0.5474321454227842</v>
       </c>
       <c r="G186" t="n">
-        <v>14.86586761329238</v>
+        <v>11.07185200162647</v>
       </c>
       <c r="H186" t="n">
         <v>0.3724250947180532</v>
@@ -6476,7 +6476,7 @@
         <v>0.5872497466304193</v>
       </c>
       <c r="G187" t="n">
-        <v>13.35934793626313</v>
+        <v>11.04260323492243</v>
       </c>
       <c r="H187" t="n">
         <v>0.3724388500065203</v>
@@ -6510,7 +6510,7 @@
         <v>0.5012011736360795</v>
       </c>
       <c r="G188" t="n">
-        <v>20.97156683268707</v>
+        <v>15.65618736580862</v>
       </c>
       <c r="H188" t="n">
         <v>0.4621166289140599</v>
@@ -6544,7 +6544,7 @@
         <v>0.5093650612289136</v>
       </c>
       <c r="G189" t="n">
-        <v>22.73665422588319</v>
+        <v>17.36776169728883</v>
       </c>
       <c r="H189" t="n">
         <v>0.4905013414818062</v>
@@ -6578,7 +6578,7 @@
         <v>0.5119216548521214</v>
       </c>
       <c r="G190" t="n">
-        <v>19.45090278605078</v>
+        <v>14.53400516181474</v>
       </c>
       <c r="H190" t="n">
         <v>0.4404274010823974</v>
@@ -6612,7 +6612,7 @@
         <v>0.4818633069605522</v>
       </c>
       <c r="G191" t="n">
-        <v>22.22321755807388</v>
+        <v>16.81048000311535</v>
       </c>
       <c r="H191" t="n">
         <v>0.4271538368011757</v>
@@ -6646,7 +6646,7 @@
         <v>0.7604243705192861</v>
       </c>
       <c r="G192" t="n">
-        <v>32.92642725428617</v>
+        <v>26.31997365636186</v>
       </c>
       <c r="H192" t="n">
         <v>0.4929931522281605</v>
@@ -6680,7 +6680,7 @@
         <v>0.7022426326260403</v>
       </c>
       <c r="G193" t="n">
-        <v>44.89908199797635</v>
+        <v>37.24684885022157</v>
       </c>
       <c r="H193" t="n">
         <v>0.4744195178683512</v>
@@ -6714,7 +6714,7 @@
         <v>0.5028185899679491</v>
       </c>
       <c r="G194" t="n">
-        <v>19.9692889012489</v>
+        <v>14.54956788569051</v>
       </c>
       <c r="H194" t="n">
         <v>0.4264943303997317</v>
@@ -6748,7 +6748,7 @@
         <v>0.5454163706047644</v>
       </c>
       <c r="G195" t="n">
-        <v>21.97884326317467</v>
+        <v>16.32083845033579</v>
       </c>
       <c r="H195" t="n">
         <v>0.3994048273772934</v>
@@ -6782,7 +6782,7 @@
         <v>0.5465768341426984</v>
       </c>
       <c r="G196" t="n">
-        <v>22.75788891459821</v>
+        <v>17.09329584641191</v>
       </c>
       <c r="H196" t="n">
         <v>0.3764550762132908</v>
@@ -6816,7 +6816,7 @@
         <v>0.5709010190806746</v>
       </c>
       <c r="G197" t="n">
-        <v>21.88193919772662</v>
+        <v>16.22848109307779</v>
       </c>
       <c r="H197" t="n">
         <v>0.472841478884683</v>
@@ -6850,7 +6850,7 @@
         <v>0.5114475504481214</v>
       </c>
       <c r="G198" t="n">
-        <v>22.79399704642027</v>
+        <v>17.16187009691918</v>
       </c>
       <c r="H198" t="n">
         <v>0.4186339250216219</v>
@@ -6884,7 +6884,7 @@
         <v>0.7287354049042202</v>
       </c>
       <c r="G199" t="n">
-        <v>33.13910216232924</v>
+        <v>26.40169993618455</v>
       </c>
       <c r="H199" t="n">
         <v>0.4978843919315616</v>
@@ -6918,7 +6918,7 @@
         <v>0.7967814147744261</v>
       </c>
       <c r="G200" t="n">
-        <v>41.7148748436983</v>
+        <v>34.45366372418451</v>
       </c>
       <c r="H200" t="n">
         <v>0.234477968686339</v>
@@ -6952,7 +6952,7 @@
         <v>0.5499370092690448</v>
       </c>
       <c r="G201" t="n">
-        <v>22.06261888481446</v>
+        <v>16.77086875201427</v>
       </c>
       <c r="H201" t="n">
         <v>0.4585821611738254</v>
@@ -6986,7 +6986,7 @@
         <v>0.5520855385497815</v>
       </c>
       <c r="G202" t="n">
-        <v>21.24346919381693</v>
+        <v>16.06886957825296</v>
       </c>
       <c r="H202" t="n">
         <v>0.4689779370969543</v>
@@ -7020,7 +7020,7 @@
         <v>0.5269664626362544</v>
       </c>
       <c r="G203" t="n">
-        <v>22.41867504135934</v>
+        <v>16.67294350378625</v>
       </c>
       <c r="H203" t="n">
         <v>0.4864509652016647</v>
@@ -7054,7 +7054,7 @@
         <v>0.5496044235166857</v>
       </c>
       <c r="G204" t="n">
-        <v>20.37528346382002</v>
+        <v>15.13162319296581</v>
       </c>
       <c r="H204" t="n">
         <v>0.4965015428096466</v>
@@ -7088,7 +7088,7 @@
         <v>0.5199292882392623</v>
       </c>
       <c r="G205" t="n">
-        <v>20.95065558767021</v>
+        <v>15.72833687991896</v>
       </c>
       <c r="H205" t="n">
         <v>0.446305084055336</v>
@@ -7122,7 +7122,7 @@
         <v>0.6000298109861018</v>
       </c>
       <c r="G206" t="n">
-        <v>31.20134752407471</v>
+        <v>24.95371210657767</v>
       </c>
       <c r="H206" t="n">
         <v>0.4632800481189601</v>
@@ -7156,7 +7156,7 @@
         <v>0.8059224748247419</v>
       </c>
       <c r="G207" t="n">
-        <v>43.28305937972697</v>
+        <v>35.93255025902445</v>
       </c>
       <c r="H207" t="n">
         <v>0.4626569831081426</v>
@@ -7190,7 +7190,7 @@
         <v>0.4889700303697877</v>
       </c>
       <c r="G208" t="n">
-        <v>21.10797728377122</v>
+        <v>15.5984450986667</v>
       </c>
       <c r="H208" t="n">
         <v>0.4532851401645291</v>
@@ -7224,7 +7224,7 @@
         <v>0.5331538985084986</v>
       </c>
       <c r="G209" t="n">
-        <v>21.76800129092254</v>
+        <v>100.0169662966697</v>
       </c>
       <c r="H209" t="n">
         <v>0.4572947282872646</v>
@@ -7258,7 +7258,7 @@
         <v>0.5433915284458547</v>
       </c>
       <c r="G210" t="n">
-        <v>22.6055706935532</v>
+        <v>17.25658582233728</v>
       </c>
       <c r="H210" t="n">
         <v>0.4313576037772059</v>
@@ -7292,7 +7292,7 @@
         <v>0.5553564981720523</v>
       </c>
       <c r="G211" t="n">
-        <v>22.34555500423765</v>
+        <v>16.91232095169868</v>
       </c>
       <c r="H211" t="n">
         <v>0.4356732184062995</v>
@@ -7326,7 +7326,7 @@
         <v>0.5132136975043283</v>
       </c>
       <c r="G212" t="n">
-        <v>22.1643239629762</v>
+        <v>16.87109513897837</v>
       </c>
       <c r="H212" t="n">
         <v>0.4707660867396724</v>
@@ -7360,7 +7360,7 @@
         <v>0.7153837838126502</v>
       </c>
       <c r="G213" t="n">
-        <v>33.88670560405717</v>
+        <v>26.82775749238238</v>
       </c>
       <c r="H213" t="n">
         <v>0.4594232240733184</v>
@@ -7394,7 +7394,7 @@
         <v>0.7513174375153199</v>
       </c>
       <c r="G214" t="n">
-        <v>42.53894018196356</v>
+        <v>35.1167683441291</v>
       </c>
       <c r="H214" t="n">
         <v>0.4850656445408728</v>
@@ -7428,7 +7428,7 @@
         <v>0.5390368774148568</v>
       </c>
       <c r="G215" t="n">
-        <v>26.90097128942018</v>
+        <v>20.81890152817447</v>
       </c>
       <c r="H215" t="n">
         <v>0.4073532088708401</v>
@@ -7462,7 +7462,7 @@
         <v>0.5273698181315475</v>
       </c>
       <c r="G216" t="n">
-        <v>21.48300217262906</v>
+        <v>16.02707463655846</v>
       </c>
       <c r="H216" t="n">
         <v>0.4356019098768433</v>
@@ -7496,7 +7496,7 @@
         <v>0.5303593721329188</v>
       </c>
       <c r="G217" t="n">
-        <v>21.56221736005566</v>
+        <v>16.36977215661602</v>
       </c>
       <c r="H217" t="n">
         <v>0.4503405445241306</v>
@@ -7530,7 +7530,7 @@
         <v>0.6029671841187828</v>
       </c>
       <c r="G218" t="n">
-        <v>18.44228381051919</v>
+        <v>15.03899469947155</v>
       </c>
       <c r="H218" t="n">
         <v>0.4119358928380596</v>
@@ -7564,7 +7564,7 @@
         <v>0.4984661204054477</v>
       </c>
       <c r="G219" t="n">
-        <v>15.4397086463702</v>
+        <v>11.37585590723906</v>
       </c>
       <c r="H219" t="n">
         <v>0.4365652596140664</v>
@@ -7598,7 +7598,7 @@
         <v>0.4630978523416195</v>
       </c>
       <c r="G220" t="n">
-        <v>16.57175968321065</v>
+        <v>12.40747682762866</v>
       </c>
       <c r="H220" t="n">
         <v>0.4514119000095582</v>
@@ -7632,7 +7632,7 @@
         <v>0.4764793276176092</v>
       </c>
       <c r="G221" t="n">
-        <v>16.26214791250969</v>
+        <v>12.13668061912238</v>
       </c>
       <c r="H221" t="n">
         <v>0.4218874440981734</v>
@@ -7666,7 +7666,7 @@
         <v>0.4800219927980968</v>
       </c>
       <c r="G222" t="n">
-        <v>16.408931868118</v>
+        <v>12.31263162316259</v>
       </c>
       <c r="H222" t="n">
         <v>0.4525406498944614</v>
@@ -7700,7 +7700,7 @@
         <v>0.6712494616592279</v>
       </c>
       <c r="G223" t="n">
-        <v>28.38828374850889</v>
+        <v>22.37692345862828</v>
       </c>
       <c r="H223" t="n">
         <v>0.4650120610401529</v>
@@ -7734,7 +7734,7 @@
         <v>0.551988322140583</v>
       </c>
       <c r="G224" t="n">
-        <v>33.80633454412097</v>
+        <v>27.55055093625039</v>
       </c>
       <c r="H224" t="n">
         <v>0.5045999164923635</v>
@@ -7768,7 +7768,7 @@
         <v>0.4851835071199125</v>
       </c>
       <c r="G225" t="n">
-        <v>16.42824382561422</v>
+        <v>12.14134845800973</v>
       </c>
       <c r="H225" t="n">
         <v>0.4199852148371497</v>
@@ -7802,7 +7802,7 @@
         <v>0.4879267197683094</v>
       </c>
       <c r="G226" t="n">
-        <v>16.0420599742431</v>
+        <v>11.89536861881492</v>
       </c>
       <c r="H226" t="n">
         <v>0.4124222144182694</v>
@@ -7836,7 +7836,7 @@
         <v>0.4939096688052749</v>
       </c>
       <c r="G227" t="n">
-        <v>17.30315824859438</v>
+        <v>12.97983783868564</v>
       </c>
       <c r="H227" t="n">
         <v>0.4110846024622523</v>
@@ -7870,7 +7870,7 @@
         <v>0.5363367001220187</v>
       </c>
       <c r="G228" t="n">
-        <v>17.46247326806164</v>
+        <v>12.88400354029404</v>
       </c>
       <c r="H228" t="n">
         <v>0.4540068349341159</v>
@@ -7904,7 +7904,7 @@
         <v>0.5026657326865663</v>
       </c>
       <c r="G229" t="n">
-        <v>16.92707586162285</v>
+        <v>12.52408015476177</v>
       </c>
       <c r="H229" t="n">
         <v>0.3909241268214004</v>
@@ -7938,7 +7938,7 @@
         <v>0.7041072364324027</v>
       </c>
       <c r="G230" t="n">
-        <v>27.46854720329644</v>
+        <v>21.5424335600696</v>
       </c>
       <c r="H230" t="n">
         <v>0.4530415472653703</v>
@@ -7972,7 +7972,7 @@
         <v>0.6778843024176765</v>
       </c>
       <c r="G231" t="n">
-        <v>34.35272861942117</v>
+        <v>27.84482047581069</v>
       </c>
       <c r="H231" t="n">
         <v>0.2053196267488685</v>
@@ -8006,7 +8006,7 @@
         <v>0.4819263599482723</v>
       </c>
       <c r="G232" t="n">
-        <v>16.01645441296555</v>
+        <v>11.88320561237464</v>
       </c>
       <c r="H232" t="n">
         <v>0.4172992238925134</v>
@@ -8040,7 +8040,7 @@
         <v>0.5274257916064721</v>
       </c>
       <c r="G233" t="n">
-        <v>15.91287096981951</v>
+        <v>11.78788618610246</v>
       </c>
       <c r="H233" t="n">
         <v>0.4618286574334311</v>
@@ -8074,7 +8074,7 @@
         <v>0.5037921972255531</v>
       </c>
       <c r="G234" t="n">
-        <v>17.6275635242588</v>
+        <v>13.31599262755274</v>
       </c>
       <c r="H234" t="n">
         <v>0.4348372769521507</v>
@@ -8108,7 +8108,7 @@
         <v>0.4969305024232101</v>
       </c>
       <c r="G235" t="n">
-        <v>15.79628294639728</v>
+        <v>11.69372211596601</v>
       </c>
       <c r="H235" t="n">
         <v>0.459322528827522</v>
@@ -8142,7 +8142,7 @@
         <v>0.5012238330209331</v>
       </c>
       <c r="G236" t="n">
-        <v>16.36847584898413</v>
+        <v>12.19293132603742</v>
       </c>
       <c r="H236" t="n">
         <v>0.4143696129058371</v>
@@ -8176,7 +8176,7 @@
         <v>0.6808580404166918</v>
       </c>
       <c r="G237" t="n">
-        <v>25.26997494642689</v>
+        <v>19.74840158664426</v>
       </c>
       <c r="H237" t="n">
         <v>0.3982495112148239</v>
@@ -8210,7 +8210,7 @@
         <v>0.6770703972785796</v>
       </c>
       <c r="G238" t="n">
-        <v>34.42769999941613</v>
+        <v>27.90847153253714</v>
       </c>
       <c r="H238" t="n">
         <v>0.4219679671752829</v>
@@ -8244,7 +8244,7 @@
         <v>0.5081027311181247</v>
       </c>
       <c r="G239" t="n">
-        <v>16.36659470470218</v>
+        <v>12.10617740734421</v>
       </c>
       <c r="H239" t="n">
         <v>0.4069727446080766</v>
@@ -8278,7 +8278,7 @@
         <v>0.5037007779083056</v>
       </c>
       <c r="G240" t="n">
-        <v>16.55679467389091</v>
+        <v>12.35071122432806</v>
       </c>
       <c r="H240" t="n">
         <v>0.4056575739377915</v>
@@ -8312,7 +8312,7 @@
         <v>0.4733662597585036</v>
       </c>
       <c r="G241" t="n">
-        <v>15.12310718977781</v>
+        <v>11.22840772758636</v>
       </c>
       <c r="H241" t="n">
         <v>0.3914956773512614</v>
@@ -8346,7 +8346,7 @@
         <v>0.4913545548926324</v>
       </c>
       <c r="G242" t="n">
-        <v>15.13039348198547</v>
+        <v>11.33874952920081</v>
       </c>
       <c r="H242" t="n">
         <v>0.4087537040397164</v>
@@ -8380,7 +8380,7 @@
         <v>0.4873396868848288</v>
       </c>
       <c r="G243" t="n">
-        <v>16.044436458474</v>
+        <v>11.56278089974779</v>
       </c>
       <c r="H243" t="n">
         <v>0.418627107441107</v>
@@ -8414,7 +8414,7 @@
         <v>0.6123999604581567</v>
       </c>
       <c r="G244" t="n">
-        <v>30.11987050720849</v>
+        <v>23.84668779833132</v>
       </c>
       <c r="H244" t="n">
         <v>0.4091118377400116</v>
@@ -8448,7 +8448,7 @@
         <v>0.9343657790381561</v>
       </c>
       <c r="G245" t="n">
-        <v>38.08818002574115</v>
+        <v>30.93317173081169</v>
       </c>
       <c r="H245" t="n">
         <v>0.4457201388214196</v>
@@ -8482,7 +8482,7 @@
         <v>0.5818164361073483</v>
       </c>
       <c r="G246" t="n">
-        <v>19.74732201189479</v>
+        <v>15.00480639991773</v>
       </c>
       <c r="H246" t="n">
         <v>0.4033672960823706</v>
@@ -8516,7 +8516,7 @@
         <v>0.4571225914222797</v>
       </c>
       <c r="G247" t="n">
-        <v>14.39096525137239</v>
+        <v>10.76468817083638</v>
       </c>
       <c r="H247" t="n">
         <v>0.4001049017866646</v>
@@ -8550,7 +8550,7 @@
         <v>0.4677857450560613</v>
       </c>
       <c r="G248" t="n">
-        <v>16.01361010725374</v>
+        <v>11.9494942328719</v>
       </c>
       <c r="H248" t="n">
         <v>0.3809346103885488</v>
@@ -8584,7 +8584,7 @@
         <v>0.5791161206843468</v>
       </c>
       <c r="G249" t="n">
-        <v>15.05159658568981</v>
+        <v>12.41449386960249</v>
       </c>
       <c r="H249" t="n">
         <v>0.413889157732122</v>
@@ -8618,7 +8618,7 @@
         <v>0.8486771776658142</v>
       </c>
       <c r="G250" t="n">
-        <v>33.89522891117422</v>
+        <v>27.21884983792017</v>
       </c>
       <c r="H250" t="n">
         <v>0.3948101187232407</v>
@@ -8652,7 +8652,7 @@
         <v>0.854006701171504</v>
       </c>
       <c r="G251" t="n">
-        <v>33.45684693496514</v>
+        <v>26.92809788562983</v>
       </c>
       <c r="H251" t="n">
         <v>0.3745205723882321</v>
@@ -8686,7 +8686,7 @@
         <v>0.7966744388943661</v>
       </c>
       <c r="G252" t="n">
-        <v>33.15265848599221</v>
+        <v>26.43087310255979</v>
       </c>
       <c r="H252" t="n">
         <v>0.3228744524136309</v>
@@ -8720,7 +8720,7 @@
         <v>0.8385506122552031</v>
       </c>
       <c r="G253" t="n">
-        <v>33.1130339214447</v>
+        <v>26.54355062496754</v>
       </c>
       <c r="H253" t="n">
         <v>0.3433448122484375</v>
@@ -8754,7 +8754,7 @@
         <v>0.8640214699320133</v>
       </c>
       <c r="G254" t="n">
-        <v>35.52546150927841</v>
+        <v>28.26374418207059</v>
       </c>
       <c r="H254" t="n">
         <v>0.3635856279759608</v>
@@ -8788,7 +8788,7 @@
         <v>0.9115555112434344</v>
       </c>
       <c r="G255" t="n">
-        <v>38.39794823358424</v>
+        <v>31.49751993040725</v>
       </c>
       <c r="H255" t="n">
         <v>0.4462434025545578</v>
@@ -8822,7 +8822,7 @@
         <v>0.858030979779118</v>
       </c>
       <c r="G256" t="n">
-        <v>34.26469682740217</v>
+        <v>27.71060942986183</v>
       </c>
       <c r="H256" t="n">
         <v>0.3885205506131597</v>
@@ -8856,7 +8856,7 @@
         <v>0.8262975432201256</v>
       </c>
       <c r="G257" t="n">
-        <v>32.63086806101747</v>
+        <v>26.23737972048814</v>
       </c>
       <c r="H257" t="n">
         <v>0.3655850913580703</v>
@@ -8890,7 +8890,7 @@
         <v>0.82754036418233</v>
       </c>
       <c r="G258" t="n">
-        <v>32.8376719358028</v>
+        <v>26.4237016922474</v>
       </c>
       <c r="H258" t="n">
         <v>0.3582985102153867</v>
@@ -8924,7 +8924,7 @@
         <v>0.851497025935917</v>
       </c>
       <c r="G259" t="n">
-        <v>32.87853125722317</v>
+        <v>26.18980250392684</v>
       </c>
       <c r="H259" t="n">
         <v>0.4061851386280272</v>
@@ -8958,7 +8958,7 @@
         <v>0.8775210494575602</v>
       </c>
       <c r="G260" t="n">
-        <v>34.59765409381325</v>
+        <v>27.67866022431521</v>
       </c>
       <c r="H260" t="n">
         <v>0.3793222703918855</v>
@@ -8992,7 +8992,7 @@
         <v>0.9499131098847801</v>
       </c>
       <c r="G261" t="n">
-        <v>36.82680539887841</v>
+        <v>29.83984566083368</v>
       </c>
       <c r="H261" t="n">
         <v>0.4097559874325143</v>
@@ -9026,7 +9026,7 @@
         <v>0.9275455561695415</v>
       </c>
       <c r="G262" t="n">
-        <v>36.15565682520235</v>
+        <v>29.15552526155537</v>
       </c>
       <c r="H262" t="n">
         <v>0.1954827764282379</v>
@@ -9060,7 +9060,7 @@
         <v>0.8844981881652224</v>
       </c>
       <c r="G263" t="n">
-        <v>34.973942978627</v>
+        <v>28.19118503178837</v>
       </c>
       <c r="H263" t="n">
         <v>0.399898299417732</v>
@@ -9094,7 +9094,7 @@
         <v>0.8953687521363909</v>
       </c>
       <c r="G264" t="n">
-        <v>35.38909421584958</v>
+        <v>28.62992943708797</v>
       </c>
       <c r="H264" t="n">
         <v>0.4311329371708257</v>
@@ -9128,7 +9128,7 @@
         <v>0.8658626661015545</v>
       </c>
       <c r="G265" t="n">
-        <v>34.61303429461895</v>
+        <v>27.77012953412607</v>
       </c>
       <c r="H265" t="n">
         <v>0.4142952311851727</v>
@@ -9162,7 +9162,7 @@
         <v>0.8722878221745658</v>
       </c>
       <c r="G266" t="n">
-        <v>34.10492732268839</v>
+        <v>27.3533124408641</v>
       </c>
       <c r="H266" t="n">
         <v>0.4190024687673531</v>
@@ -9196,7 +9196,7 @@
         <v>0.8912176920660047</v>
       </c>
       <c r="G267" t="n">
-        <v>34.59196704966119</v>
+        <v>27.82314746971312</v>
       </c>
       <c r="H267" t="n">
         <v>0.3969251517625028</v>
@@ -9230,7 +9230,7 @@
         <v>0.9135630420997315</v>
       </c>
       <c r="G268" t="n">
-        <v>35.90488826219069</v>
+        <v>29.20559751062232</v>
       </c>
       <c r="H268" t="n">
         <v>0.4195348719195328</v>
@@ -9264,7 +9264,7 @@
         <v>0.9138391583533844</v>
       </c>
       <c r="G269" t="n">
-        <v>36.50504004143102</v>
+        <v>29.74491925394151</v>
       </c>
       <c r="H269" t="n">
         <v>0.4653783994112006</v>
@@ -9298,7 +9298,7 @@
         <v>0.8519231891144851</v>
       </c>
       <c r="G270" t="n">
-        <v>34.04207091660955</v>
+        <v>27.34026447817818</v>
       </c>
       <c r="H270" t="n">
         <v>0.4468474757298437</v>
@@ -9332,7 +9332,7 @@
         <v>0.8569194166185479</v>
       </c>
       <c r="G271" t="n">
-        <v>34.53604327063138</v>
+        <v>27.7335178635611</v>
       </c>
       <c r="H271" t="n">
         <v>0.4411134721658618</v>
@@ -9366,7 +9366,7 @@
         <v>0.8780521518909423</v>
       </c>
       <c r="G272" t="n">
-        <v>34.26695562293097</v>
+        <v>27.49807942534463</v>
       </c>
       <c r="H272" t="n">
         <v>0.4124235282636202</v>
@@ -9400,7 +9400,7 @@
         <v>0.9074157792582661</v>
       </c>
       <c r="G273" t="n">
-        <v>34.56320551009544</v>
+        <v>27.76098388665309</v>
       </c>
       <c r="H273" t="n">
         <v>0.4160848454181224</v>
@@ -9434,7 +9434,7 @@
         <v>0.8894033315144974</v>
       </c>
       <c r="G274" t="n">
-        <v>35.09670688508226</v>
+        <v>28.27922065992649</v>
       </c>
       <c r="H274" t="n">
         <v>0.4347038607705251</v>
@@ -9468,7 +9468,7 @@
         <v>0.8869367326544659</v>
       </c>
       <c r="G275" t="n">
-        <v>36.539182850112</v>
+        <v>29.50435714163647</v>
       </c>
       <c r="H275" t="n">
         <v>0.4019229542932246</v>
@@ -9502,7 +9502,7 @@
         <v>0.951971708032488</v>
       </c>
       <c r="G276" t="n">
-        <v>37.22701976099393</v>
+        <v>30.22034989163268</v>
       </c>
       <c r="H276" t="n">
         <v>0.4322315994270587</v>
@@ -9536,7 +9536,7 @@
         <v>0.8784818491419397</v>
       </c>
       <c r="G277" t="n">
-        <v>34.85919068622793</v>
+        <v>27.8901554850826</v>
       </c>
       <c r="H277" t="n">
         <v>0.371465981276522</v>
@@ -9570,7 +9570,7 @@
         <v>0.9028473765923887</v>
       </c>
       <c r="G278" t="n">
-        <v>34.69463214546121</v>
+        <v>27.74174563979633</v>
       </c>
       <c r="H278" t="n">
         <v>0.3661624448187862</v>
@@ -9604,7 +9604,7 @@
         <v>0.8658064933250642</v>
       </c>
       <c r="G279" t="n">
-        <v>34.50549625553285</v>
+        <v>27.82355581898141</v>
       </c>
       <c r="H279" t="n">
         <v>0.3554329307730388</v>
@@ -9638,7 +9638,7 @@
         <v>0.8821127717508729</v>
       </c>
       <c r="G280" t="n">
-        <v>34.70419055482799</v>
+        <v>31.47147605583448</v>
       </c>
       <c r="H280" t="n">
         <v>0.3403406035829502</v>
@@ -9672,7 +9672,7 @@
         <v>0.5107271484837237</v>
       </c>
       <c r="G281" t="n">
-        <v>19.64611733034306</v>
+        <v>15.31439153262763</v>
       </c>
       <c r="H281" t="n">
         <v>0.2317272803251676</v>
@@ -9706,7 +9706,7 @@
         <v>0.4645335646769165</v>
       </c>
       <c r="G282" t="n">
-        <v>17.62064804069011</v>
+        <v>13.27380818681062</v>
       </c>
       <c r="H282" t="n">
         <v>0.2148862877156944</v>
@@ -9740,7 +9740,7 @@
         <v>0.4605810411021408</v>
       </c>
       <c r="G283" t="n">
-        <v>19.86990196192388</v>
+        <v>15.11890804278013</v>
       </c>
       <c r="H283" t="n">
         <v>0.1594193392582947</v>
@@ -9774,7 +9774,7 @@
         <v>0.5135853892417132</v>
       </c>
       <c r="G284" t="n">
-        <v>19.04635171175947</v>
+        <v>14.61149482376615</v>
       </c>
       <c r="H284" t="n">
         <v>0.2056100848940089</v>
@@ -9808,7 +9808,7 @@
         <v>0.5195772502297218</v>
       </c>
       <c r="G285" t="n">
-        <v>26.48198676294752</v>
+        <v>20.74913305902841</v>
       </c>
       <c r="H285" t="n">
         <v>0.2717675590665284</v>
@@ -9842,7 +9842,7 @@
         <v>0.8250281809763167</v>
       </c>
       <c r="G286" t="n">
-        <v>36.94712205307236</v>
+        <v>29.91418652197889</v>
       </c>
       <c r="H286" t="n">
         <v>0.3035547480011779</v>
@@ -9876,7 +9876,7 @@
         <v>0.5280248203361146</v>
       </c>
       <c r="G287" t="n">
-        <v>20.27804196046346</v>
+        <v>15.05059227940977</v>
       </c>
       <c r="H287" t="n">
         <v>0.203358812397303</v>
@@ -9910,7 +9910,7 @@
         <v>0.5225834502419188</v>
       </c>
       <c r="G288" t="n">
-        <v>20.41436153397058</v>
+        <v>15.76939970355428</v>
       </c>
       <c r="H288" t="n">
         <v>0.1699194503354187</v>
@@ -9944,7 +9944,7 @@
         <v>0.4921871574223051</v>
       </c>
       <c r="G289" t="n">
-        <v>18.97873074805598</v>
+        <v>14.364263407361</v>
       </c>
       <c r="H289" t="n">
         <v>0.1490000912243384</v>
@@ -9978,7 +9978,7 @@
         <v>0.5854242902571478</v>
       </c>
       <c r="G290" t="n">
-        <v>21.61592849480484</v>
+        <v>16.96239816169049</v>
       </c>
       <c r="H290" t="n">
         <v>0.2083131432370475</v>
@@ -10012,7 +10012,7 @@
         <v>0.4395324141685975</v>
       </c>
       <c r="G291" t="n">
-        <v>19.80717492432603</v>
+        <v>15.29340887418975</v>
       </c>
       <c r="H291" t="n">
         <v>0.1846084653240589</v>
@@ -10046,7 +10046,7 @@
         <v>0.5594421880020648</v>
       </c>
       <c r="G292" t="n">
-        <v>29.99780347760828</v>
+        <v>23.73443883392765</v>
       </c>
       <c r="H292" t="n">
         <v>0.2649092555213847</v>
@@ -10080,7 +10080,7 @@
         <v>0.7938178623779663</v>
       </c>
       <c r="G293" t="n">
-        <v>35.91231936098789</v>
+        <v>29.01154920621625</v>
       </c>
       <c r="H293" t="n">
         <v>0.07747430592435998</v>
@@ -10114,7 +10114,7 @@
         <v>0.5418663998949661</v>
       </c>
       <c r="G294" t="n">
-        <v>21.86059718236396</v>
+        <v>16.00934858896724</v>
       </c>
       <c r="H294" t="n">
         <v>0.2158327257891469</v>
@@ -10148,7 +10148,7 @@
         <v>0.5207315506126899</v>
       </c>
       <c r="G295" t="n">
-        <v>20.51055756406026</v>
+        <v>16.07114810221812</v>
       </c>
       <c r="H295" t="n">
         <v>0.2225034749174196</v>
@@ -10182,7 +10182,7 @@
         <v>0.5349302792586884</v>
       </c>
       <c r="G296" t="n">
-        <v>21.06449409829577</v>
+        <v>16.62647069540831</v>
       </c>
       <c r="H296" t="n">
         <v>0.2001349988927472</v>
@@ -10216,7 +10216,7 @@
         <v>0.5226028329924155</v>
       </c>
       <c r="G297" t="n">
-        <v>21.17142931122416</v>
+        <v>15.88977418696186</v>
       </c>
       <c r="H297" t="n">
         <v>0.1973483880557768</v>
@@ -10250,7 +10250,7 @@
         <v>0.4560343873986145</v>
       </c>
       <c r="G298" t="n">
-        <v>16.76541003302344</v>
+        <v>13.2691576544375</v>
       </c>
       <c r="H298" t="n">
         <v>0.1762024875009796</v>
@@ -10284,7 +10284,7 @@
         <v>0.6135035075986894</v>
       </c>
       <c r="G299" t="n">
-        <v>27.24382406545561</v>
+        <v>21.39723584016555</v>
       </c>
       <c r="H299" t="n">
         <v>0.2351144431593269</v>
@@ -10318,7 +10318,7 @@
         <v>0.8072439527655603</v>
       </c>
       <c r="G300" t="n">
-        <v>34.38758769854591</v>
+        <v>27.87414626538594</v>
       </c>
       <c r="H300" t="n">
         <v>0.3077646803055142</v>
@@ -10352,7 +10352,7 @@
         <v>0.4677583521169473</v>
       </c>
       <c r="G301" t="n">
-        <v>19.33359268028077</v>
+        <v>14.74846582426318</v>
       </c>
       <c r="H301" t="n">
         <v>0.204099385274478</v>
@@ -10386,7 +10386,7 @@
         <v>0.4741384243078405</v>
       </c>
       <c r="G302" t="n">
-        <v>18.7893340229964</v>
+        <v>14.47899106066454</v>
       </c>
       <c r="H302" t="n">
         <v>0.2290748645501572</v>
@@ -10420,7 +10420,7 @@
         <v>0.5213420577830391</v>
       </c>
       <c r="G303" t="n">
-        <v>20.68481768825175</v>
+        <v>16.33518934304834</v>
       </c>
       <c r="H303" t="n">
         <v>0.1920203988604381</v>
@@ -10454,7 +10454,7 @@
         <v>0.5174319836508271</v>
       </c>
       <c r="G304" t="n">
-        <v>21.2738203035101</v>
+        <v>15.95487406467431</v>
       </c>
       <c r="H304" t="n">
         <v>0.1749703586390135</v>
@@ -10488,7 +10488,7 @@
         <v>0.4911572095461608</v>
       </c>
       <c r="G305" t="n">
-        <v>20.36602307721503</v>
+        <v>15.96450336944519</v>
       </c>
       <c r="H305" t="n">
         <v>0.1824533529277289</v>
@@ -10522,7 +10522,7 @@
         <v>0.6006574655717769</v>
       </c>
       <c r="G306" t="n">
-        <v>23.67093415859997</v>
+        <v>18.51749516120339</v>
       </c>
       <c r="H306" t="n">
         <v>0.211911570861931</v>
@@ -10556,7 +10556,7 @@
         <v>0.8869472767315685</v>
       </c>
       <c r="G307" t="n">
-        <v>38.30223806984204</v>
+        <v>31.38247795863897</v>
       </c>
       <c r="H307" t="n">
         <v>0.1622510081566342</v>
@@ -10590,7 +10590,7 @@
         <v>0.5047640325875706</v>
       </c>
       <c r="G308" t="n">
-        <v>20.01884373624258</v>
+        <v>15.51380231832175</v>
       </c>
       <c r="H308" t="n">
         <v>0.1888743963180818</v>
@@ -10624,7 +10624,7 @@
         <v>0.4883501616471441</v>
       </c>
       <c r="G309" t="n">
-        <v>15.90046785545708</v>
+        <v>12.10574554831067</v>
       </c>
       <c r="H309" t="n">
         <v>0.2056285220062203</v>
@@ -10658,7 +10658,7 @@
         <v>0.5009403707716606</v>
       </c>
       <c r="G310" t="n">
-        <v>19.00192429130952</v>
+        <v>14.95331998747441</v>
       </c>
       <c r="H310" t="n">
         <v>0.1847641098735304</v>
@@ -10692,7 +10692,7 @@
         <v>0.5711037706544317</v>
       </c>
       <c r="G311" t="n">
-        <v>18.12154507942869</v>
+        <v>15.86441982724781</v>
       </c>
       <c r="H311" t="n">
         <v>0.1550183726005303</v>
@@ -10726,7 +10726,7 @@
         <v>0.2512088189349099</v>
       </c>
       <c r="G312" t="n">
-        <v>12.85870415866323</v>
+        <v>6.602649829362034</v>
       </c>
       <c r="H312" t="n">
         <v>0.3064934951074728</v>
@@ -10760,7 +10760,7 @@
         <v>0.2389410283847887</v>
       </c>
       <c r="G313" t="n">
-        <v>11.07467054303303</v>
+        <v>5.775761033855253</v>
       </c>
       <c r="H313" t="n">
         <v>0.3113976184634992</v>
@@ -10794,7 +10794,7 @@
         <v>0.2778490836313499</v>
       </c>
       <c r="G314" t="n">
-        <v>10.79657013828898</v>
+        <v>5.395937164329758</v>
       </c>
       <c r="H314" t="n">
         <v>0.2757483525880827</v>
@@ -10828,7 +10828,7 @@
         <v>0.3859538116826756</v>
       </c>
       <c r="G315" t="n">
-        <v>9.018696891369983</v>
+        <v>6.949775725038548</v>
       </c>
       <c r="H315" t="n">
         <v>0.2910021932197582</v>
@@ -10862,7 +10862,7 @@
         <v>0.2907767831084916</v>
       </c>
       <c r="G316" t="n">
-        <v>26.840568041226</v>
+        <v>31.26305267990682</v>
       </c>
       <c r="H316" t="n">
         <v>0.3134280500151441</v>
@@ -10896,7 +10896,7 @@
         <v>0.2102616124918172</v>
       </c>
       <c r="G317" t="n">
-        <v>44.75016357776244</v>
+        <v>31.36609291542216</v>
       </c>
       <c r="H317" t="n">
         <v>0.3623519211877902</v>
@@ -10930,7 +10930,7 @@
         <v>0.3478404315435482</v>
       </c>
       <c r="G318" t="n">
-        <v>23.24325905600851</v>
+        <v>10.52100069368504</v>
       </c>
       <c r="H318" t="n">
         <v>0.2937370811267606</v>
@@ -10964,7 +10964,7 @@
         <v>0.2779022232236095</v>
       </c>
       <c r="G319" t="n">
-        <v>20.24195704168939</v>
+        <v>7.83416971375688</v>
       </c>
       <c r="H319" t="n">
         <v>0.2710036357041812</v>
@@ -10998,7 +10998,7 @@
         <v>0.2167511020944527</v>
       </c>
       <c r="G320" t="n">
-        <v>13.44824128663511</v>
+        <v>13.11304092841479</v>
       </c>
       <c r="H320" t="n">
         <v>0.2759468469931219</v>
@@ -11032,7 +11032,7 @@
         <v>0.3760325292300464</v>
       </c>
       <c r="G321" t="n">
-        <v>15.86875252019853</v>
+        <v>6.68241399976204</v>
       </c>
       <c r="H321" t="n">
         <v>0.330179921492625</v>
@@ -11066,7 +11066,7 @@
         <v>0.2445020568663155</v>
       </c>
       <c r="G322" t="n">
-        <v>9.485712764655958</v>
+        <v>6.201844688033449</v>
       </c>
       <c r="H322" t="n">
         <v>0.2621996676284666</v>
@@ -11100,7 +11100,7 @@
         <v>0.5644737118680579</v>
       </c>
       <c r="G323" t="n">
-        <v>37.18460775238495</v>
+        <v>29.57909183699065</v>
       </c>
       <c r="H323" t="n">
         <v>0.3155466862125447</v>
@@ -11134,7 +11134,7 @@
         <v>0.2275116672733582</v>
       </c>
       <c r="G324" t="n">
-        <v>40.65191895750898</v>
+        <v>2.646497862550278</v>
       </c>
       <c r="H324" t="n">
         <v>0.09226271065961927</v>
@@ -11168,7 +11168,7 @@
         <v>0.2554075985761329</v>
       </c>
       <c r="G325" t="n">
-        <v>8.311512395886934</v>
+        <v>5.187869567140467</v>
       </c>
       <c r="H325" t="n">
         <v>0.2775525721797517</v>
@@ -11202,7 +11202,7 @@
         <v>0.2493769027545836</v>
       </c>
       <c r="G326" t="n">
-        <v>13.75602444365212</v>
+        <v>6.397642868715272</v>
       </c>
       <c r="H326" t="n">
         <v>0.309747094433826</v>
@@ -11236,7 +11236,7 @@
         <v>0.2473390033509216</v>
       </c>
       <c r="G327" t="n">
-        <v>4.434600803636806</v>
+        <v>4.525692885680879</v>
       </c>
       <c r="H327" t="n">
         <v>0.2902330780764976</v>
@@ -11270,7 +11270,7 @@
         <v>0.3573188931413683</v>
       </c>
       <c r="G328" t="n">
-        <v>20.87755770896457</v>
+        <v>9.292467645723109</v>
       </c>
       <c r="H328" t="n">
         <v>0.3034780961758167</v>
@@ -11304,7 +11304,7 @@
         <v>0.2615570568864216</v>
       </c>
       <c r="G329" t="n">
-        <v>10.41113705521399</v>
+        <v>8.240014434848927</v>
       </c>
       <c r="H329" t="n">
         <v>0.2707176543610253</v>
@@ -11338,7 +11338,7 @@
         <v>0.661852709172418</v>
       </c>
       <c r="G330" t="n">
-        <v>22.75340023399695</v>
+        <v>22.53975406553088</v>
       </c>
       <c r="H330" t="n">
         <v>0.3103521286261414</v>
@@ -11372,7 +11372,7 @@
         <v>0.2461733724352257</v>
       </c>
       <c r="G331" t="n">
-        <v>38.0514484381746</v>
+        <v>26.1667661942899</v>
       </c>
       <c r="H331" t="n">
         <v>0.3537970522951244</v>
@@ -11406,7 +11406,7 @@
         <v>0.2181223797223631</v>
       </c>
       <c r="G332" t="n">
-        <v>7.700541275606483</v>
+        <v>5.592162010824632</v>
       </c>
       <c r="H332" t="n">
         <v>0.3118350281575002</v>
@@ -11440,7 +11440,7 @@
         <v>0.2293711326615225</v>
       </c>
       <c r="G333" t="n">
-        <v>7.905876556094111</v>
+        <v>5.66511170805401</v>
       </c>
       <c r="H333" t="n">
         <v>0.3221536940382374</v>
@@ -11474,7 +11474,7 @@
         <v>0.2896251016259764</v>
       </c>
       <c r="G334" t="n">
-        <v>18.24294693384007</v>
+        <v>10.20032034994025</v>
       </c>
       <c r="H334" t="n">
         <v>0.2965271704596892</v>
@@ -11508,7 +11508,7 @@
         <v>0.3613130589189197</v>
       </c>
       <c r="G335" t="n">
-        <v>14.34337551101397</v>
+        <v>9.440671217482853</v>
       </c>
       <c r="H335" t="n">
         <v>0.3135309054295451</v>
@@ -11542,7 +11542,7 @@
         <v>0.4193274396298945</v>
       </c>
       <c r="G336" t="n">
-        <v>23.69690680435181</v>
+        <v>16.53419887420433</v>
       </c>
       <c r="H336" t="n">
         <v>0.3287842708845661</v>
@@ -11576,7 +11576,7 @@
         <v>0.6051453921724883</v>
       </c>
       <c r="G337" t="n">
-        <v>22.51417584523757</v>
+        <v>26.0068149368397</v>
       </c>
       <c r="H337" t="n">
         <v>0.3143149214114223</v>
@@ -11610,7 +11610,7 @@
         <v>0.2213651787049339</v>
       </c>
       <c r="G338" t="n">
-        <v>41.21310598101484</v>
+        <v>36.35631442856438</v>
       </c>
       <c r="H338" t="n">
         <v>0.3558147997530159</v>
@@ -11644,7 +11644,7 @@
         <v>0.3837890883652313</v>
       </c>
       <c r="G339" t="n">
-        <v>15.61953857490076</v>
+        <v>9.558682740297563</v>
       </c>
       <c r="H339" t="n">
         <v>0.3079690149762999</v>
@@ -11678,7 +11678,7 @@
         <v>0.2322412876272421</v>
       </c>
       <c r="G340" t="n">
-        <v>7.84128407359832</v>
+        <v>5.27002205644657</v>
       </c>
       <c r="H340" t="n">
         <v>0.3030582268821165</v>
@@ -11712,7 +11712,7 @@
         <v>0.4120000912330334</v>
       </c>
       <c r="G341" t="n">
-        <v>21.88582225521947</v>
+        <v>9.14865379426011</v>
       </c>
       <c r="H341" t="n">
         <v>0.3012936339387081</v>
@@ -11746,7 +11746,7 @@
         <v>0.5594587261627938</v>
       </c>
       <c r="G342" t="n">
-        <v>11.36566143912692</v>
+        <v>6.512100523392811</v>
       </c>
       <c r="H342" t="n">
         <v>0.2879695181703519</v>
@@ -11780,7 +11780,7 @@
         <v>0.4382376728010478</v>
       </c>
       <c r="G343" t="n">
-        <v>19.0665682746247</v>
+        <v>15.13706604925647</v>
       </c>
       <c r="H343" t="n">
         <v>0.467842428839393</v>
@@ -11814,7 +11814,7 @@
         <v>0.3761331801549874</v>
       </c>
       <c r="G344" t="n">
-        <v>21.14541170942726</v>
+        <v>16.45810824086252</v>
       </c>
       <c r="H344" t="n">
         <v>0.4767623870368917</v>
@@ -11848,7 +11848,7 @@
         <v>0.4070082293662166</v>
       </c>
       <c r="G345" t="n">
-        <v>12.92887820352606</v>
+        <v>10.57789408865542</v>
       </c>
       <c r="H345" t="n">
         <v>0.4442158177356419</v>
@@ -11882,7 +11882,7 @@
         <v>0.4531686172161652</v>
       </c>
       <c r="G346" t="n">
-        <v>27.65271988430132</v>
+        <v>22.40036906278374</v>
       </c>
       <c r="H346" t="n">
         <v>0.440085634522487</v>
@@ -11916,7 +11916,7 @@
         <v>0.4868429868345912</v>
       </c>
       <c r="G347" t="n">
-        <v>34.86682367734304</v>
+        <v>33.09229974027753</v>
       </c>
       <c r="H347" t="n">
         <v>0.436468876590501</v>
@@ -11950,7 +11950,7 @@
         <v>0.8588795127454568</v>
       </c>
       <c r="G348" t="n">
-        <v>36.35291675053372</v>
+        <v>29.90785733983203</v>
       </c>
       <c r="H348" t="n">
         <v>0.4579501579539194</v>
@@ -11984,7 +11984,7 @@
         <v>0.4651867542773205</v>
       </c>
       <c r="G349" t="n">
-        <v>25.3738930306998</v>
+        <v>20.72033563292526</v>
       </c>
       <c r="H349" t="n">
         <v>0.4575381852921116</v>
@@ -12018,7 +12018,7 @@
         <v>0.401835329782823</v>
       </c>
       <c r="G350" t="n">
-        <v>13.66724493136036</v>
+        <v>11.14518779610855</v>
       </c>
       <c r="H350" t="n">
         <v>0.4406896734083537</v>
@@ -12052,7 +12052,7 @@
         <v>0.3564583650334093</v>
       </c>
       <c r="G351" t="n">
-        <v>24.04001185092347</v>
+        <v>19.75015184276234</v>
       </c>
       <c r="H351" t="n">
         <v>0.4267289333715904</v>
@@ -12086,7 +12086,7 @@
         <v>0.3987602889885402</v>
       </c>
       <c r="G352" t="n">
-        <v>13.84954540848387</v>
+        <v>9.82729072616884</v>
       </c>
       <c r="H352" t="n">
         <v>0.4916987518974584</v>
@@ -12120,7 +12120,7 @@
         <v>0.3403702330181099</v>
       </c>
       <c r="G353" t="n">
-        <v>19.41306937924787</v>
+        <v>14.84453306104364</v>
       </c>
       <c r="H353" t="n">
         <v>0.4450893600809763</v>
@@ -12154,7 +12154,7 @@
         <v>0.5212843148395406</v>
       </c>
       <c r="G354" t="n">
-        <v>34.73782878266822</v>
+        <v>33.16437183897177</v>
       </c>
       <c r="H354" t="n">
         <v>0.4689919793663246</v>
@@ -12188,7 +12188,7 @@
         <v>0.8086520250037432</v>
       </c>
       <c r="G355" t="n">
-        <v>36.30550620436379</v>
+        <v>29.23221886760002</v>
       </c>
       <c r="H355" t="n">
         <v>0.1994919867245838</v>
@@ -12222,7 +12222,7 @@
         <v>0.3516220836960167</v>
       </c>
       <c r="G356" t="n">
-        <v>28.80845098888094</v>
+        <v>28.25421766457162</v>
       </c>
       <c r="H356" t="n">
         <v>0.439420381254134</v>
@@ -12256,7 +12256,7 @@
         <v>0.3925700826077249</v>
       </c>
       <c r="G357" t="n">
-        <v>10.12546397945222</v>
+        <v>3.431160133922689</v>
       </c>
       <c r="H357" t="n">
         <v>0.4495836076811179</v>
@@ -12290,7 +12290,7 @@
         <v>0.3724935862290439</v>
       </c>
       <c r="G358" t="n">
-        <v>14.98716160477358</v>
+        <v>8.854111556368718</v>
       </c>
       <c r="H358" t="n">
         <v>0.3873426201899253</v>
@@ -12324,7 +12324,7 @@
         <v>0.3772233594242614</v>
       </c>
       <c r="G359" t="n">
-        <v>9.813930467708845</v>
+        <v>4.507854692176296</v>
       </c>
       <c r="H359" t="n">
         <v>0.4798077903318118</v>
@@ -12358,7 +12358,7 @@
         <v>0.4061650690017779</v>
       </c>
       <c r="G360" t="n">
-        <v>18.70838116452403</v>
+        <v>14.50218465398533</v>
       </c>
       <c r="H360" t="n">
         <v>0.4459030399793676</v>
@@ -12392,7 +12392,7 @@
         <v>0.6384551946602829</v>
       </c>
       <c r="G361" t="n">
-        <v>38.99938444206582</v>
+        <v>37.13598990450928</v>
       </c>
       <c r="H361" t="n">
         <v>0.4098318666561369</v>
@@ -12426,7 +12426,7 @@
         <v>0.7349976922653908</v>
       </c>
       <c r="G362" t="n">
-        <v>34.1491386191828</v>
+        <v>27.42612185749838</v>
       </c>
       <c r="H362" t="n">
         <v>0.4370548346626621</v>
@@ -12460,7 +12460,7 @@
         <v>0.3517968257750284</v>
       </c>
       <c r="G363" t="n">
-        <v>21.07798460763524</v>
+        <v>17.49264077066297</v>
       </c>
       <c r="H363" t="n">
         <v>0.468181839855376</v>
@@ -12494,7 +12494,7 @@
         <v>0.3221922934380204</v>
       </c>
       <c r="G364" t="n">
-        <v>12.2545220393971</v>
+        <v>10.41650912836239</v>
       </c>
       <c r="H364" t="n">
         <v>0.4856834550536251</v>
@@ -12528,7 +12528,7 @@
         <v>0.5012652140110431</v>
       </c>
       <c r="G365" t="n">
-        <v>22.21152223401672</v>
+        <v>17.1395113177646</v>
       </c>
       <c r="H365" t="n">
         <v>0.4792845360774405</v>
@@ -12562,7 +12562,7 @@
         <v>0.4115035095480351</v>
       </c>
       <c r="G366" t="n">
-        <v>16.04653533847492</v>
+        <v>11.87730255666234</v>
       </c>
       <c r="H366" t="n">
         <v>0.4582091173560419</v>
@@ -12596,7 +12596,7 @@
         <v>0.3584894359550165</v>
       </c>
       <c r="G367" t="n">
-        <v>26.65723601242903</v>
+        <v>22.07298343296744</v>
       </c>
       <c r="H367" t="n">
         <v>0.4753936416023778</v>
@@ -12630,7 +12630,7 @@
         <v>0.5901932569319203</v>
       </c>
       <c r="G368" t="n">
-        <v>33.8168966442441</v>
+        <v>37.23392289502032</v>
       </c>
       <c r="H368" t="n">
         <v>0.416252688530057</v>
@@ -12664,7 +12664,7 @@
         <v>0.8076167142497174</v>
       </c>
       <c r="G369" t="n">
-        <v>38.72241841119454</v>
+        <v>31.50169184225384</v>
       </c>
       <c r="H369" t="n">
         <v>0.4552741590506367</v>
@@ -12698,7 +12698,7 @@
         <v>0.4110692866968873</v>
       </c>
       <c r="G370" t="n">
-        <v>24.33117359677791</v>
+        <v>21.3992636113897</v>
       </c>
       <c r="H370" t="n">
         <v>0.4685465119755119</v>
@@ -12732,7 +12732,7 @@
         <v>0.3596921021667543</v>
       </c>
       <c r="G371" t="n">
-        <v>17.6329026027605</v>
+        <v>17.09122423285715</v>
       </c>
       <c r="H371" t="n">
         <v>0.467073223982468</v>
@@ -12766,7 +12766,7 @@
         <v>0.4347426862293229</v>
       </c>
       <c r="G372" t="n">
-        <v>29.74582266340785</v>
+        <v>23.16144972002527</v>
       </c>
       <c r="H372" t="n">
         <v>0.4318383937240834</v>
@@ -12800,7 +12800,7 @@
         <v>0.4792084599772158</v>
       </c>
       <c r="G373" t="n">
-        <v>28.01634378535736</v>
+        <v>0</v>
       </c>
       <c r="H373" t="n">
         <v>0.4792147280632169</v>
@@ -12834,7 +12834,7 @@
         <v>0.5432318945649448</v>
       </c>
       <c r="G374" t="n">
-        <v>20.66571705255685</v>
+        <v>15.72000165855845</v>
       </c>
       <c r="H374" t="n">
         <v>0.2596837329079342</v>
@@ -12868,7 +12868,7 @@
         <v>0.5593616964865108</v>
       </c>
       <c r="G375" t="n">
-        <v>20.1793025563217</v>
+        <v>15.4116182300169</v>
       </c>
       <c r="H375" t="n">
         <v>0.2610461003629658</v>
@@ -12902,7 +12902,7 @@
         <v>0.5391113976285801</v>
       </c>
       <c r="G376" t="n">
-        <v>21.48661583878916</v>
+        <v>16.70230889662016</v>
       </c>
       <c r="H376" t="n">
         <v>0.272046513165113</v>
@@ -12936,7 +12936,7 @@
         <v>0.5628488327881402</v>
       </c>
       <c r="G377" t="n">
-        <v>22.09148190077518</v>
+        <v>16.72225596525241</v>
       </c>
       <c r="H377" t="n">
         <v>0.2838665916813288</v>
@@ -12970,7 +12970,7 @@
         <v>0.5650697730834295</v>
       </c>
       <c r="G378" t="n">
-        <v>26.9365267447748</v>
+        <v>21.38244447670543</v>
       </c>
       <c r="H378" t="n">
         <v>0.3066069538198401</v>
@@ -13004,7 +13004,7 @@
         <v>0.8173093358045281</v>
       </c>
       <c r="G379" t="n">
-        <v>39.52362327396738</v>
+        <v>31.83948953761094</v>
       </c>
       <c r="H379" t="n">
         <v>0.3481695042002491</v>
@@ -13038,7 +13038,7 @@
         <v>0.6011026389207085</v>
       </c>
       <c r="G380" t="n">
-        <v>23.148633410505</v>
+        <v>17.73224281676528</v>
       </c>
       <c r="H380" t="n">
         <v>0.2619028565787684</v>
@@ -13072,7 +13072,7 @@
         <v>0.647715277865567</v>
       </c>
       <c r="G381" t="n">
-        <v>25.18518578808882</v>
+        <v>19.21653098619082</v>
       </c>
       <c r="H381" t="n">
         <v>0.2167971598348849</v>
@@ -13106,7 +13106,7 @@
         <v>0.6925009118927087</v>
       </c>
       <c r="G382" t="n">
-        <v>25.64760980886838</v>
+        <v>19.92957089882931</v>
       </c>
       <c r="H382" t="n">
         <v>0.2104199905445276</v>
@@ -13140,7 +13140,7 @@
         <v>0.6564580014563396</v>
       </c>
       <c r="G383" t="n">
-        <v>24.47211298390631</v>
+        <v>18.46030196677883</v>
       </c>
       <c r="H383" t="n">
         <v>0.2169134584206322</v>
@@ -13174,7 +13174,7 @@
         <v>0.6090289227046722</v>
       </c>
       <c r="G384" t="n">
-        <v>24.08751344055877</v>
+        <v>18.23597653333742</v>
       </c>
       <c r="H384" t="n">
         <v>0.2531892542463323</v>
@@ -13208,7 +13208,7 @@
         <v>0.5147664741698528</v>
       </c>
       <c r="G385" t="n">
-        <v>26.99003268846084</v>
+        <v>21.71600975255861</v>
       </c>
       <c r="H385" t="n">
         <v>0.3064517744843673</v>
@@ -13242,7 +13242,7 @@
         <v>0.9172172241763332</v>
       </c>
       <c r="G386" t="n">
-        <v>38.67610600604669</v>
+        <v>31.47685723059244</v>
       </c>
       <c r="H386" t="n">
         <v>0.0858480048285183</v>
@@ -13276,7 +13276,7 @@
         <v>0.6676988661799059</v>
       </c>
       <c r="G387" t="n">
-        <v>23.65069442016742</v>
+        <v>17.63042788366075</v>
       </c>
       <c r="H387" t="n">
         <v>0.2792012237362902</v>
@@ -13310,7 +13310,7 @@
         <v>0.6405765628748794</v>
       </c>
       <c r="G388" t="n">
-        <v>24.75100377828437</v>
+        <v>18.69123275589154</v>
       </c>
       <c r="H388" t="n">
         <v>0.210824941246414</v>
@@ -13344,7 +13344,7 @@
         <v>0.6214932265721672</v>
       </c>
       <c r="G389" t="n">
-        <v>22.29447586465327</v>
+        <v>16.96082784471225</v>
       </c>
       <c r="H389" t="n">
         <v>0.2430069602018604</v>
@@ -13378,7 +13378,7 @@
         <v>0.6469083184726092</v>
       </c>
       <c r="G390" t="n">
-        <v>21.94988545979392</v>
+        <v>16.8274090229731</v>
       </c>
       <c r="H390" t="n">
         <v>0.301690598736943</v>
@@ -13412,7 +13412,7 @@
         <v>0.63954887814297</v>
       </c>
       <c r="G391" t="n">
-        <v>21.92296421750997</v>
+        <v>16.32282714506465</v>
       </c>
       <c r="H391" t="n">
         <v>0.2987093414005076</v>
@@ -13446,7 +13446,7 @@
         <v>0.6653157395311635</v>
       </c>
       <c r="G392" t="n">
-        <v>27.28844651348055</v>
+        <v>20.73795359403115</v>
       </c>
       <c r="H392" t="n">
         <v>0.244275822394789</v>
@@ -13480,7 +13480,7 @@
         <v>0.6836076785435675</v>
       </c>
       <c r="G393" t="n">
-        <v>41.92431943372156</v>
+        <v>34.6380113415125</v>
       </c>
       <c r="H393" t="n">
         <v>0.3236804834937603</v>
@@ -13514,7 +13514,7 @@
         <v>0.6043031119109805</v>
       </c>
       <c r="G394" t="n">
-        <v>21.95477996721825</v>
+        <v>16.83420787088323</v>
       </c>
       <c r="H394" t="n">
         <v>0.2378370157599627</v>
@@ -13548,7 +13548,7 @@
         <v>0.6113291697018491</v>
       </c>
       <c r="G395" t="n">
-        <v>23.02583953359588</v>
+        <v>18.01180323400181</v>
       </c>
       <c r="H395" t="n">
         <v>0.2272005953449071</v>
@@ -13582,7 +13582,7 @@
         <v>0.6223455927950017</v>
       </c>
       <c r="G396" t="n">
-        <v>21.05645868466903</v>
+        <v>16.46960218226011</v>
       </c>
       <c r="H396" t="n">
         <v>0.206561660074203</v>
@@ -13616,7 +13616,7 @@
         <v>0.631478157227348</v>
       </c>
       <c r="G397" t="n">
-        <v>22.59876645388031</v>
+        <v>16.97160393980757</v>
       </c>
       <c r="H397" t="n">
         <v>0.2713550669524754</v>
@@ -13650,7 +13650,7 @@
         <v>0.5860370739625331</v>
       </c>
       <c r="G398" t="n">
-        <v>22.34968612553538</v>
+        <v>16.43679412569677</v>
       </c>
       <c r="H398" t="n">
         <v>0.2648872545816789</v>
@@ -13684,7 +13684,7 @@
         <v>0.5700366098099803</v>
       </c>
       <c r="G399" t="n">
-        <v>25.76192458741002</v>
+        <v>19.83648120171153</v>
       </c>
       <c r="H399" t="n">
         <v>0.2571041376820939</v>
@@ -13718,7 +13718,7 @@
         <v>0.8112144709664028</v>
       </c>
       <c r="G400" t="n">
-        <v>39.92946305236114</v>
+        <v>32.30430862126003</v>
       </c>
       <c r="H400" t="n">
         <v>0.3560908911829062</v>
@@ -13752,7 +13752,7 @@
         <v>0.6035728328732802</v>
       </c>
       <c r="G401" t="n">
-        <v>23.95783991111282</v>
+        <v>18.54039566074297</v>
       </c>
       <c r="H401" t="n">
         <v>0.2309775445849929</v>
@@ -13786,7 +13786,7 @@
         <v>0.6564555976419988</v>
       </c>
       <c r="G402" t="n">
-        <v>23.96003261854009</v>
+        <v>18.5131894312095</v>
       </c>
       <c r="H402" t="n">
         <v>0.1951689881267632</v>
@@ -13820,7 +13820,7 @@
         <v>0.5658805041915207</v>
       </c>
       <c r="G403" t="n">
-        <v>22.96426927019687</v>
+        <v>17.72676064088273</v>
       </c>
       <c r="H403" t="n">
         <v>0.2945884980027563</v>
@@ -13854,7 +13854,7 @@
         <v>0.5914688360649168</v>
       </c>
       <c r="G404" t="n">
-        <v>19.70025904358789</v>
+        <v>16.99490377356689</v>
       </c>
       <c r="H404" t="n">
         <v>0.2165077114016619</v>
@@ -13888,7 +13888,7 @@
         <v>0.6617352871130753</v>
       </c>
       <c r="G405" t="n">
-        <v>20.5882697648348</v>
+        <v>15.85670053859366</v>
       </c>
       <c r="H405" t="n">
         <v>0.349405910804044</v>
@@ -13922,7 +13922,7 @@
         <v>0.6063910563667203</v>
       </c>
       <c r="G406" t="n">
-        <v>19.80804246308651</v>
+        <v>14.91445978076798</v>
       </c>
       <c r="H406" t="n">
         <v>0.3474893436832384</v>
@@ -13956,7 +13956,7 @@
         <v>0.6349657980888441</v>
       </c>
       <c r="G407" t="n">
-        <v>20.79369574319458</v>
+        <v>15.84631820106426</v>
       </c>
       <c r="H407" t="n">
         <v>0.3050763385799571</v>
@@ -13990,7 +13990,7 @@
         <v>0.6474872231801032</v>
       </c>
       <c r="G408" t="n">
-        <v>22.26225284636816</v>
+        <v>17.04578059326606</v>
       </c>
       <c r="H408" t="n">
         <v>0.339365341911557</v>
@@ -14024,7 +14024,7 @@
         <v>0.5194238839224402</v>
       </c>
       <c r="G409" t="n">
-        <v>27.4022458605566</v>
+        <v>22.19718366520606</v>
       </c>
       <c r="H409" t="n">
         <v>0.3419944078393213</v>
@@ -14058,7 +14058,7 @@
         <v>0.9434468880709346</v>
       </c>
       <c r="G410" t="n">
-        <v>38.98646669196496</v>
+        <v>31.69643617993923</v>
       </c>
       <c r="H410" t="n">
         <v>0.3676459732610393</v>
@@ -14092,7 +14092,7 @@
         <v>0.5761067102696689</v>
       </c>
       <c r="G411" t="n">
-        <v>18.96474082984285</v>
+        <v>14.1295721155453</v>
       </c>
       <c r="H411" t="n">
         <v>0.323445751831734</v>
@@ -14126,7 +14126,7 @@
         <v>0.6586849338865612</v>
       </c>
       <c r="G412" t="n">
-        <v>19.6612363825559</v>
+        <v>14.91783282369427</v>
       </c>
       <c r="H412" t="n">
         <v>0.3197759250622812</v>
@@ -14160,7 +14160,7 @@
         <v>0.6503015862921707</v>
       </c>
       <c r="G413" t="n">
-        <v>20.0856474657787</v>
+        <v>15.28175516392738</v>
       </c>
       <c r="H413" t="n">
         <v>0.3021395689257981</v>
@@ -14194,7 +14194,7 @@
         <v>0.6457389254593572</v>
       </c>
       <c r="G414" t="n">
-        <v>19.63615318823322</v>
+        <v>15.15208264350665</v>
       </c>
       <c r="H414" t="n">
         <v>0.3707675107432594</v>
@@ -14228,7 +14228,7 @@
         <v>0.6352076443376694</v>
       </c>
       <c r="G415" t="n">
-        <v>22.91351082262904</v>
+        <v>17.45146973510059</v>
       </c>
       <c r="H415" t="n">
         <v>0.2983672524591791</v>
@@ -14262,7 +14262,7 @@
         <v>0.5677533978137633</v>
       </c>
       <c r="G416" t="n">
-        <v>22.1647286291157</v>
+        <v>17.58608602936507</v>
       </c>
       <c r="H416" t="n">
         <v>0.3397991160430296</v>
@@ -14296,7 +14296,7 @@
         <v>0.757682797243822</v>
       </c>
       <c r="G417" t="n">
-        <v>23.50940545411816</v>
+        <v>18.44455385905558</v>
       </c>
       <c r="H417" t="n">
         <v>0.1356267646191077</v>
@@ -14330,7 +14330,7 @@
         <v>0.632420261326919</v>
       </c>
       <c r="G418" t="n">
-        <v>19.70354370104782</v>
+        <v>14.88088168182291</v>
       </c>
       <c r="H418" t="n">
         <v>0.3017262553908718</v>
@@ -14364,7 +14364,7 @@
         <v>0.6644040039573189</v>
       </c>
       <c r="G419" t="n">
-        <v>20.35147158119998</v>
+        <v>15.45841589918378</v>
       </c>
       <c r="H419" t="n">
         <v>0.3528769555128066</v>
@@ -14398,7 +14398,7 @@
         <v>0.6677792792723782</v>
       </c>
       <c r="G420" t="n">
-        <v>20.78898402298078</v>
+        <v>15.75492607824012</v>
       </c>
       <c r="H420" t="n">
         <v>0.3354844353986481</v>
@@ -14432,7 +14432,7 @@
         <v>0.6004496932944079</v>
       </c>
       <c r="G421" t="n">
-        <v>20.09897542581401</v>
+        <v>15.51214532760211</v>
       </c>
       <c r="H421" t="n">
         <v>0.3522547829658498</v>
@@ -14466,7 +14466,7 @@
         <v>0.6316986128716643</v>
       </c>
       <c r="G422" t="n">
-        <v>20.23702275991479</v>
+        <v>15.268698723165</v>
       </c>
       <c r="H422" t="n">
         <v>0.3278344222509742</v>
@@ -14500,7 +14500,7 @@
         <v>0.5494271587770371</v>
       </c>
       <c r="G423" t="n">
-        <v>20.38664666063345</v>
+        <v>16.1312326768266</v>
       </c>
       <c r="H423" t="n">
         <v>0.3592950807758189</v>
@@ -14534,7 +14534,7 @@
         <v>0.7124110926072004</v>
       </c>
       <c r="G424" t="n">
-        <v>23.37488025104745</v>
+        <v>18.17492895909536</v>
       </c>
       <c r="H424" t="n">
         <v>0.392963664347421</v>
@@ -14568,7 +14568,7 @@
         <v>0.6043995444040371</v>
       </c>
       <c r="G425" t="n">
-        <v>18.30158299060059</v>
+        <v>13.62898683049364</v>
       </c>
       <c r="H425" t="n">
         <v>0.3767253589368467</v>
@@ -14602,7 +14602,7 @@
         <v>0.6298386425836339</v>
       </c>
       <c r="G426" t="n">
-        <v>18.37044685049092</v>
+        <v>13.85637823871959</v>
       </c>
       <c r="H426" t="n">
         <v>0.3803139592392259</v>
@@ -14636,7 +14636,7 @@
         <v>0.6204743271764763</v>
       </c>
       <c r="G427" t="n">
-        <v>18.34413586163601</v>
+        <v>13.62421995805793</v>
       </c>
       <c r="H427" t="n">
         <v>0.3438964354813538</v>
@@ -14670,7 +14670,7 @@
         <v>0.640882305771874</v>
       </c>
       <c r="G428" t="n">
-        <v>18.77889463755194</v>
+        <v>14.24541866470994</v>
       </c>
       <c r="H428" t="n">
         <v>0.367950661360571</v>
@@ -14704,7 +14704,7 @@
         <v>0.6191695432807686</v>
       </c>
       <c r="G429" t="n">
-        <v>19.53777028603355</v>
+        <v>14.4827485209346</v>
       </c>
       <c r="H429" t="n">
         <v>0.3835980124402686</v>
@@ -14738,7 +14738,7 @@
         <v>0.5413670877736736</v>
       </c>
       <c r="G430" t="n">
-        <v>25.84761209995931</v>
+        <v>20.21135423915476</v>
       </c>
       <c r="H430" t="n">
         <v>0.3493686094386191</v>
@@ -14772,7 +14772,7 @@
         <v>0.8822762355274034</v>
       </c>
       <c r="G431" t="n">
-        <v>39.30314040863433</v>
+        <v>32.03968148121854</v>
       </c>
       <c r="H431" t="n">
         <v>0.3792549968824399</v>
@@ -14806,7 +14806,7 @@
         <v>0.6412584102391843</v>
       </c>
       <c r="G432" t="n">
-        <v>19.32773556442532</v>
+        <v>14.57181471099041</v>
       </c>
       <c r="H432" t="n">
         <v>0.3452022431103514</v>
@@ -14840,7 +14840,7 @@
         <v>0.6195124384476713</v>
       </c>
       <c r="G433" t="n">
-        <v>19.42027878311194</v>
+        <v>14.67284585906486</v>
       </c>
       <c r="H433" t="n">
         <v>0.3649271595975752</v>
@@ -14874,7 +14874,7 @@
         <v>0.6429458390277002</v>
       </c>
       <c r="G434" t="n">
-        <v>18.87953964946508</v>
+        <v>0.1766727017302403</v>
       </c>
       <c r="H434" t="n">
         <v>0.3560234926826873</v>
@@ -14908,7 +14908,7 @@
         <v>0.6300556511000202</v>
       </c>
       <c r="G435" t="n">
-        <v>17.63018311700899</v>
+        <v>14.94980655326959</v>
       </c>
       <c r="H435" t="n">
         <v>0.3697937970617678</v>
@@ -14942,7 +14942,7 @@
         <v>0.592111460231828</v>
       </c>
       <c r="G436" t="n">
-        <v>18.46506503752118</v>
+        <v>13.84771260351009</v>
       </c>
       <c r="H436" t="n">
         <v>0.3331977093702663</v>
@@ -14976,7 +14976,7 @@
         <v>0.5392545451208426</v>
       </c>
       <c r="G437" t="n">
-        <v>18.33978412339704</v>
+        <v>13.52371705564895</v>
       </c>
       <c r="H437" t="n">
         <v>0.3295195875420451</v>
@@ -15010,7 +15010,7 @@
         <v>0.4315494527253254</v>
       </c>
       <c r="G438" t="n">
-        <v>19.64008016743933</v>
+        <v>15.43298261948459</v>
       </c>
       <c r="H438" t="n">
         <v>0.2767536089996494</v>
@@ -15044,7 +15044,7 @@
         <v>0.4916889390442565</v>
       </c>
       <c r="G439" t="n">
-        <v>21.64723848117849</v>
+        <v>17.02242018661916</v>
       </c>
       <c r="H439" t="n">
         <v>0.3251934802748274</v>
@@ -15078,7 +15078,7 @@
         <v>0.4487586406710782</v>
       </c>
       <c r="G440" t="n">
-        <v>21.62890029591122</v>
+        <v>17.34683440120523</v>
       </c>
       <c r="H440" t="n">
         <v>0.3556546579114967</v>
@@ -15112,7 +15112,7 @@
         <v>0.8376726431612679</v>
       </c>
       <c r="G441" t="n">
-        <v>36.62899226093364</v>
+        <v>29.82749957107921</v>
       </c>
       <c r="H441" t="n">
         <v>0.424702577679658</v>
@@ -15146,7 +15146,7 @@
         <v>0.5678761613726683</v>
       </c>
       <c r="G442" t="n">
-        <v>20.74158915811525</v>
+        <v>15.51818257587343</v>
       </c>
       <c r="H442" t="n">
         <v>0.359424714604693</v>
@@ -15180,7 +15180,7 @@
         <v>0.5398536810102184</v>
       </c>
       <c r="G443" t="n">
-        <v>18.40277715527005</v>
+        <v>14.26291027701725</v>
       </c>
       <c r="H443" t="n">
         <v>0.3138741739380791</v>
@@ -15214,7 +15214,7 @@
         <v>0.505223546808113</v>
       </c>
       <c r="G444" t="n">
-        <v>16.395977459824</v>
+        <v>12.28359846525415</v>
       </c>
       <c r="H444" t="n">
         <v>0.3017207451459177</v>
@@ -15248,7 +15248,7 @@
         <v>0.5304912199268301</v>
       </c>
       <c r="G445" t="n">
-        <v>17.19620322100176</v>
+        <v>13.73011536226778</v>
       </c>
       <c r="H445" t="n">
         <v>0.3584556891164727</v>
@@ -15282,7 +15282,7 @@
         <v>0.4739776781313045</v>
       </c>
       <c r="G446" t="n">
-        <v>13.50229083530096</v>
+        <v>10.42991879641387</v>
       </c>
       <c r="H446" t="n">
         <v>0.2711287546501186</v>
@@ -15316,7 +15316,7 @@
         <v>0.4869238827092842</v>
       </c>
       <c r="G447" t="n">
-        <v>19.7752266742226</v>
+        <v>15.38673370727906</v>
       </c>
       <c r="H447" t="n">
         <v>0.3547647332646429</v>
@@ -15350,7 +15350,7 @@
         <v>0.562034201048767</v>
       </c>
       <c r="G448" t="n">
-        <v>31.25330054844858</v>
+        <v>25.25840013092141</v>
       </c>
       <c r="H448" t="n">
         <v>0.1346156712336935</v>
@@ -15384,7 +15384,7 @@
         <v>0.5309434837997065</v>
       </c>
       <c r="G449" t="n">
-        <v>19.69887857587417</v>
+        <v>14.49360894530035</v>
       </c>
       <c r="H449" t="n">
         <v>0.3283237921393208</v>
@@ -15418,7 +15418,7 @@
         <v>0.4716248986512395</v>
       </c>
       <c r="G450" t="n">
-        <v>18.72042457269856</v>
+        <v>14.24967177691497</v>
       </c>
       <c r="H450" t="n">
         <v>0.343963240111274</v>
@@ -15452,7 +15452,7 @@
         <v>0.5122924493083812</v>
       </c>
       <c r="G451" t="n">
-        <v>21.12979707266457</v>
+        <v>16.10839113620543</v>
       </c>
       <c r="H451" t="n">
         <v>0.322714781805417</v>
@@ -15486,7 +15486,7 @@
         <v>0.5221438409333875</v>
       </c>
       <c r="G452" t="n">
-        <v>16.40364245338919</v>
+        <v>12.53547634135932</v>
       </c>
       <c r="H452" t="n">
         <v>0.2978942509742831</v>
@@ -15520,7 +15520,7 @@
         <v>0.5488436419230827</v>
       </c>
       <c r="G453" t="n">
-        <v>16.37023206439298</v>
+        <v>13.00923136017714</v>
       </c>
       <c r="H453" t="n">
         <v>0.2564223618600941</v>
@@ -15554,7 +15554,7 @@
         <v>0.4654711118214728</v>
       </c>
       <c r="G454" t="n">
-        <v>17.23861771764697</v>
+        <v>12.9649307820941</v>
       </c>
       <c r="H454" t="n">
         <v>0.3154201104484173</v>
@@ -15588,7 +15588,7 @@
         <v>0.708983481520409</v>
       </c>
       <c r="G455" t="n">
-        <v>29.44145859466265</v>
+        <v>23.32724540413319</v>
       </c>
       <c r="H455" t="n">
         <v>0.3829792947378889</v>
@@ -15622,7 +15622,7 @@
         <v>0.4901304055678258</v>
       </c>
       <c r="G456" t="n">
-        <v>16.84493361852863</v>
+        <v>12.7993014928654</v>
       </c>
       <c r="H456" t="n">
         <v>0.3313392539471923</v>
@@ -15656,7 +15656,7 @@
         <v>0.526210175565575</v>
       </c>
       <c r="G457" t="n">
-        <v>17.10609402413988</v>
+        <v>12.96741345515535</v>
       </c>
       <c r="H457" t="n">
         <v>0.3496296563344646</v>
@@ -15690,7 +15690,7 @@
         <v>0.5708616668669892</v>
       </c>
       <c r="G458" t="n">
-        <v>17.171014066456</v>
+        <v>12.47539957331983</v>
       </c>
       <c r="H458" t="n">
         <v>0.3371911495496335</v>
@@ -15724,7 +15724,7 @@
         <v>0.5475792029782234</v>
       </c>
       <c r="G459" t="n">
-        <v>16.46389438944014</v>
+        <v>12.40486239158942</v>
       </c>
       <c r="H459" t="n">
         <v>0.3354983541721976</v>
@@ -15758,7 +15758,7 @@
         <v>0.5227252217830165</v>
       </c>
       <c r="G460" t="n">
-        <v>15.43947270353712</v>
+        <v>11.95266465427908</v>
       </c>
       <c r="H460" t="n">
         <v>0.3649051321145563</v>
@@ -15792,7 +15792,7 @@
         <v>0.4978179743164354</v>
       </c>
       <c r="G461" t="n">
-        <v>14.2916204328965</v>
+        <v>10.49939327890028</v>
       </c>
       <c r="H461" t="n">
         <v>0.3386920404602762</v>
@@ -15826,7 +15826,7 @@
         <v>0.8635065770684087</v>
       </c>
       <c r="G462" t="n">
-        <v>38.20186059280646</v>
+        <v>31.57317936786728</v>
       </c>
       <c r="H462" t="n">
         <v>0.424452440429628</v>
@@ -15860,7 +15860,7 @@
         <v>0.4097826491157223</v>
       </c>
       <c r="G463" t="n">
-        <v>12.97390184740385</v>
+        <v>9.276995230394764</v>
       </c>
       <c r="H463" t="n">
         <v>0.3422560897949347</v>
@@ -15894,7 +15894,7 @@
         <v>0.4496684167721388</v>
       </c>
       <c r="G464" t="n">
-        <v>14.24611055241756</v>
+        <v>10.72163828626513</v>
       </c>
       <c r="H464" t="n">
         <v>0.3322193343307212</v>
@@ -15928,7 +15928,7 @@
         <v>0.5093423347709453</v>
       </c>
       <c r="G465" t="n">
-        <v>15.82801280422233</v>
+        <v>11.5233952037117</v>
       </c>
       <c r="H465" t="n">
         <v>0.3138988899400347</v>
@@ -15962,7 +15962,7 @@
         <v>0.6100840599115658</v>
       </c>
       <c r="G466" t="n">
-        <v>18.80168039534094</v>
+        <v>15.95543316039366</v>
       </c>
       <c r="H466" t="n">
         <v>0.2973055681114082</v>

</xml_diff>